<commit_message>
Modificacion historias de usuarios y product Backlong
</commit_message>
<xml_diff>
--- a/Docs/Proyecto.xlsx
+++ b/Docs/Proyecto.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PERSONAL\Desktop\Universidad\Sexto semestre 2026 - I\Ingeneria de software II\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PERSONAL\Desktop\Universidad\Sexto semestre 2026 - I\Ingeneria de software II\AsistenteVirtual\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4B22D5A-872F-41DD-BAA2-D3BC0B411ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E2FDE4A-B034-4469-A741-9B53DDAD7AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Épicas" sheetId="7" r:id="rId1"/>
@@ -23,7 +23,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="6">Ejemplo!$A$1:$K$10</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Historias de Usuario'!$A$4:$K$40</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Historias de Usuario'!$A$4:$K$37</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">Instructivo!$A$1:$D$14</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="233">
   <si>
     <t>Desarrollo ágil: Historias de usuario y criterios de aceptación</t>
   </si>
@@ -86,79 +86,16 @@
     <t>Como un usuario con discapacidad auditiva</t>
   </si>
   <si>
-    <t>Explicación de contenido</t>
-  </si>
-  <si>
-    <t>En caso que el usuario esté navegando en una página con información compleja</t>
-  </si>
-  <si>
-    <t>cuando active el asistente virtual</t>
-  </si>
-  <si>
-    <t>el sistema muestra una explicación simplificada del contenido</t>
-  </si>
-  <si>
-    <t>Activación del asistente</t>
-  </si>
-  <si>
-    <t>En caso que el usuario necesite ayuda para entender la página</t>
-  </si>
-  <si>
-    <t>cuando presione el botón del asistente</t>
-  </si>
-  <si>
-    <t>el sistema despliega la ayuda visual</t>
-  </si>
-  <si>
     <t>HU-0002</t>
   </si>
   <si>
-    <t>Inicio del trámite</t>
-  </si>
-  <si>
-    <t>En caso que el usuario ingrese a un trámite digital</t>
-  </si>
-  <si>
-    <t>cuando active la guía del asistente</t>
-  </si>
-  <si>
-    <t>el sistema muestra los pasos necesarios para completar el trámite</t>
-  </si>
-  <si>
-    <t>Avance en el proceso</t>
-  </si>
-  <si>
-    <t>En caso que el usuario complete un paso</t>
-  </si>
-  <si>
-    <t>cuando presione continuar</t>
-  </si>
-  <si>
-    <t>el sistema muestra el siguiente paso del proceso</t>
-  </si>
-  <si>
     <t>HU-0003</t>
   </si>
   <si>
     <t>Confirmación exitosa</t>
   </si>
   <si>
-    <t>En caso que el usuario complete una acción en la página</t>
-  </si>
-  <si>
-    <t>cuando envíe un formulario</t>
-  </si>
-  <si>
-    <t>el sistema muestra un mensaje visual indicando que el proceso fue exitoso</t>
-  </si>
-  <si>
     <t>Error en el proceso</t>
-  </si>
-  <si>
-    <t>En caso que exista un error en la información ingresada</t>
-  </si>
-  <si>
-    <t>cuando el usuario intente continuar</t>
   </si>
   <si>
     <t>el sistema muestra un mensaje visual indicando el error</t>
@@ -351,66 +288,12 @@
     <t>Alta</t>
   </si>
   <si>
-    <t>Quiero que el asistente virtual simplifique el contenido de la página web</t>
-  </si>
-  <si>
-    <t>Como un usuario de una plataforma web institucional con discapacidad visual</t>
-  </si>
-  <si>
-    <t>Mostrar confirmación visual al usuario</t>
-  </si>
-  <si>
     <t>HU-0004</t>
   </si>
   <si>
-    <t>Quiero activar el asistente virtual desde cualquier página</t>
-  </si>
-  <si>
-    <t>para realizar procesos en línea sin dificultad</t>
-  </si>
-  <si>
-    <t>Quiero recibir una guía paso a paso para completar un trámite</t>
-  </si>
-  <si>
-    <t>para comprender fácilmente la información y los trámites digitales</t>
-  </si>
-  <si>
-    <t>Quiero recibir mensajes visuales de confirmación</t>
-  </si>
-  <si>
-    <t>para saber si una acción se realizó correctamente</t>
-  </si>
-  <si>
-    <t>para recibir ayuda cunado la necesite</t>
-  </si>
-  <si>
-    <t>cuando presione el botón de activación</t>
-  </si>
-  <si>
-    <t>el sistema activa el asistente virtual y muestra las opciones de ayuda disponibles</t>
-  </si>
-  <si>
-    <t>En caso de que el usuario se encuentre navegando en cualquier sección del sitio web</t>
-  </si>
-  <si>
-    <t>Asistencia disponible en todas las páginas</t>
-  </si>
-  <si>
-    <t>En caso de que el usuario cambie o navegue a otra página dentro del sitio web</t>
-  </si>
-  <si>
-    <t>cuando el usuario presiones nuevamente el botón del asistente</t>
-  </si>
-  <si>
-    <t>el sistema mantiene disponible el asistente virrual y permite al usuario acceder a sus funciones de ayuda</t>
-  </si>
-  <si>
     <t>HU0004</t>
   </si>
   <si>
-    <t>Activar asistente virtual desde cualquier página</t>
-  </si>
-  <si>
     <t>Matriz Stakeholders</t>
   </si>
   <si>
@@ -483,162 +366,27 @@
     <t>HU-0008</t>
   </si>
   <si>
-    <t>HU-0009</t>
-  </si>
-  <si>
     <t>Como usuario con discapacidad auditiva</t>
   </si>
   <si>
-    <t>quiero convertir voz a texto</t>
-  </si>
-  <si>
-    <t>para comprender fácilmente el contenido del sitio web</t>
-  </si>
-  <si>
-    <t>En caso que el sisitema detecte audio</t>
-  </si>
-  <si>
-    <t>cuando el usuario active la función de conversión de voz</t>
-  </si>
-  <si>
-    <t>el sistema convierte la voz en texto visible en la pantalla</t>
-  </si>
-  <si>
-    <t>Convertir voz a texto</t>
-  </si>
-  <si>
-    <t>Visualización del texto</t>
-  </si>
-  <si>
-    <t>en caso de que el sistema haya convetido el audio a texto</t>
-  </si>
-  <si>
-    <t>cuando el sistema procese el audio</t>
-  </si>
-  <si>
-    <t>el sistema muestra el texto generado</t>
-  </si>
-  <si>
-    <t>quiero traducir texto a lengua de signos colombiana</t>
-  </si>
-  <si>
-    <t>para poder comprender mejor la información de la página web</t>
-  </si>
-  <si>
-    <t>Traducción del contenido</t>
-  </si>
-  <si>
-    <t>En caso de que el usario ingrese en la página</t>
-  </si>
-  <si>
-    <t>cuando el usuario active la función de traducción a señas</t>
-  </si>
-  <si>
-    <t>el sistema muestra una representación en lengua de señas colombiana</t>
-  </si>
-  <si>
     <t>Reproducción de señas</t>
   </si>
   <si>
-    <t>En caso de que el sistema haya generado una traducción</t>
-  </si>
-  <si>
-    <t>cuando el usuario presione reproducir</t>
-  </si>
-  <si>
-    <t>el sistema reproduce la interpretación visual en lengua de señas colombiana</t>
-  </si>
-  <si>
     <t>quiero recibir alertas visuales</t>
   </si>
   <si>
-    <t>para identificar eventos importantes dentro del sistema</t>
-  </si>
-  <si>
     <t>Notificación visual</t>
   </si>
   <si>
-    <t>En caso que ocurra un evento importante deltro del sisitema</t>
-  </si>
-  <si>
-    <t>cuando el sistema detcte el evento</t>
-  </si>
-  <si>
     <t>el sistema muestra una alerta visual</t>
   </si>
   <si>
     <t>Confirmación de alaerta</t>
   </si>
   <si>
-    <t>En caso que el usuario vea la alerta en pantalla</t>
-  </si>
-  <si>
     <t>cuando el usuario presione aceptar</t>
   </si>
   <si>
-    <t>el sisitema cierra la alerta</t>
-  </si>
-  <si>
-    <t>Como un usuario con dispacacidad auditiva</t>
-  </si>
-  <si>
-    <t>Quiero recibir indicaciones sobre el siguiente paso</t>
-  </si>
-  <si>
-    <t>para completar correctamente los trámites en línea</t>
-  </si>
-  <si>
-    <t>Identificación del paso actual</t>
-  </si>
-  <si>
-    <t>En caso que el usuario se encuentre realizando un trámite</t>
-  </si>
-  <si>
-    <t>cuando el usuario complete el paso a paso</t>
-  </si>
-  <si>
-    <t>el sistema indicara el siguiente paso del proceso</t>
-  </si>
-  <si>
-    <t>Guía del proceso</t>
-  </si>
-  <si>
-    <t>En caso que el sistema identifique el siguiente paso</t>
-  </si>
-  <si>
-    <t>cuando el sisitema muestre la guía</t>
-  </si>
-  <si>
-    <t>el sistema muestra instrucciones del paso a continuar</t>
-  </si>
-  <si>
-    <t>para personalizar el uso del asistente según mis necesidades</t>
-  </si>
-  <si>
-    <t>Activación de funciones</t>
-  </si>
-  <si>
-    <t>En caso que el usuario acceda a la configuración del asistente</t>
-  </si>
-  <si>
-    <t>cuando el usuario active una función</t>
-  </si>
-  <si>
-    <t>el sistema habilita la función</t>
-  </si>
-  <si>
-    <t>Desactivación de funciones</t>
-  </si>
-  <si>
-    <t>En caso que el usuario tenga funciones activadas</t>
-  </si>
-  <si>
-    <t>cuando el usuario desactive una función</t>
-  </si>
-  <si>
-    <t>el sistema deshabilita la función seleccionada.</t>
-  </si>
-  <si>
     <t>HU0005</t>
   </si>
   <si>
@@ -651,37 +399,7 @@
     <t>HU0008</t>
   </si>
   <si>
-    <t>HU0009</t>
-  </si>
-  <si>
-    <t>configurar las funciones del asistente</t>
-  </si>
-  <si>
-    <t>Simplificar el contenido de la página web mediante el asisitente</t>
-  </si>
-  <si>
-    <t>Proporcionar una guía paso a paso para completar los trámites digitales</t>
-  </si>
-  <si>
-    <t>Convertir voz a texto para comprensión del usuario</t>
-  </si>
-  <si>
-    <t>Traducir texto a lenguaje de signos</t>
-  </si>
-  <si>
-    <t>Indicar el siguiente paso en el proceso digital</t>
-  </si>
-  <si>
-    <t>Configurar las funciones del asistente virtual</t>
-  </si>
-  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>Baja</t>
-  </si>
-  <si>
-    <t>Mostrar alertas visuales cuando haya un evento importante</t>
   </si>
   <si>
     <t>Fase</t>
@@ -785,6 +503,255 @@
 CAD: Ingeniería de Software II
 Universidad de Cundinamarca
 </t>
+  </si>
+  <si>
+    <t>Quiero quela extension detecte automaticamente texto, audio o video en una página</t>
+  </si>
+  <si>
+    <t>para poder acceder a su contenido en formato accedible</t>
+  </si>
+  <si>
+    <t>Detección de texto</t>
+  </si>
+  <si>
+    <t>En caso que el usuario esté navegando en una página web</t>
+  </si>
+  <si>
+    <t>cuando la extensión se active</t>
+  </si>
+  <si>
+    <t>el sistema identifica el contenido textual</t>
+  </si>
+  <si>
+    <t>Detección multimedia</t>
+  </si>
+  <si>
+    <t>En caso que existan audios o videos</t>
+  </si>
+  <si>
+    <t>cuando la página cargue</t>
+  </si>
+  <si>
+    <t>el sistema identifica contenido multimedia</t>
+  </si>
+  <si>
+    <t>quiero convertir el texto de la página a lengua de señas colombiana</t>
+  </si>
+  <si>
+    <t>para comprender la información</t>
+  </si>
+  <si>
+    <t>Traducción de texto</t>
+  </si>
+  <si>
+    <t>En caso de que exista contenido textual</t>
+  </si>
+  <si>
+    <t>cuando el usuario active la función</t>
+  </si>
+  <si>
+    <t>el sistema muestra una avatar interprete de LSC</t>
+  </si>
+  <si>
+    <t>En caso de exista una traducción</t>
+  </si>
+  <si>
+    <t>cuando el usuario interactue</t>
+  </si>
+  <si>
+    <t>el sistema reproduce la interpretación visual en LSC</t>
+  </si>
+  <si>
+    <t>Como un usuario con discapacidad auditiva que sabe leer</t>
+  </si>
+  <si>
+    <t>Quiero convertir audio o video a texto</t>
+  </si>
+  <si>
+    <t>para  entender el contenido multimedia</t>
+  </si>
+  <si>
+    <t>Detección de audio o video</t>
+  </si>
+  <si>
+    <t>En caso que exista contenido multimedia</t>
+  </si>
+  <si>
+    <t>el sistema procesa el audio</t>
+  </si>
+  <si>
+    <t>Generación de texto</t>
+  </si>
+  <si>
+    <t>En caso que el audio sea procesado</t>
+  </si>
+  <si>
+    <t>cuando finalice el procesamiento</t>
+  </si>
+  <si>
+    <t>el sistema muestra la transcripción en pantalla</t>
+  </si>
+  <si>
+    <t>para entender el estado de las acciones</t>
+  </si>
+  <si>
+    <t>cuando falle el proceso</t>
+  </si>
+  <si>
+    <t>Quiero convertir audio o video en LSC</t>
+  </si>
+  <si>
+    <t>para comprender el contenido sin necesidad de leer</t>
+  </si>
+  <si>
+    <t>Procesamiento multimedia</t>
+  </si>
+  <si>
+    <t>En caso que exista audio/video</t>
+  </si>
+  <si>
+    <t>cuando el audio active la función</t>
+  </si>
+  <si>
+    <t>el sistema interpreta el contenido</t>
+  </si>
+  <si>
+    <t>Representación en LSC</t>
+  </si>
+  <si>
+    <t>En caso de que el contenido sea procesado</t>
+  </si>
+  <si>
+    <t>cuando se genere la salida</t>
+  </si>
+  <si>
+    <t>el sistema muestra una interpretación en LSC</t>
+  </si>
+  <si>
+    <t>Quiero activar la extensión desde cualquier página</t>
+  </si>
+  <si>
+    <t>para acceder a sus funcionalidades</t>
+  </si>
+  <si>
+    <t>Activación</t>
+  </si>
+  <si>
+    <t>En caso de que el usuario navegue</t>
+  </si>
+  <si>
+    <t>cuando presione el icono de extensión</t>
+  </si>
+  <si>
+    <t>el sistema habilita las funciones</t>
+  </si>
+  <si>
+    <t>Persistencia</t>
+  </si>
+  <si>
+    <t>En caso de que cambie de página web</t>
+  </si>
+  <si>
+    <t>cuando la extensión esté activada</t>
+  </si>
+  <si>
+    <t>el sistema mantiene su funcionamiento</t>
+  </si>
+  <si>
+    <t>Quiero recibir confirmaciónes visuales en LSC</t>
+  </si>
+  <si>
+    <t>En caso que el usuario complete una acción</t>
+  </si>
+  <si>
+    <t>cuando el proceso finalice</t>
+  </si>
+  <si>
+    <t>el sistema muestra una confirmación visual o en LSC</t>
+  </si>
+  <si>
+    <t>En caso que ocurra un error</t>
+  </si>
+  <si>
+    <t>para identificar eventos importantes</t>
+  </si>
+  <si>
+    <t>En caso que ocurra un evento importante dentro del sistema</t>
+  </si>
+  <si>
+    <t>cuando el sistema detecte</t>
+  </si>
+  <si>
+    <t>En caso que el usuario interactúe</t>
+  </si>
+  <si>
+    <t>el sistema cierra la alerta</t>
+  </si>
+  <si>
+    <t>configurar si prefiero texto o LSC</t>
+  </si>
+  <si>
+    <t>para personalizar mi experiencia según mis condiciones</t>
+  </si>
+  <si>
+    <t>Configuración</t>
+  </si>
+  <si>
+    <t>Aplicación</t>
+  </si>
+  <si>
+    <t>En caso que el usuario acceda a la configuración</t>
+  </si>
+  <si>
+    <t>cuando seleccione preferencia</t>
+  </si>
+  <si>
+    <t>el sistema guarda la configuración</t>
+  </si>
+  <si>
+    <t>En caso que el usuario navegue</t>
+  </si>
+  <si>
+    <t>cuando use la extensión</t>
+  </si>
+  <si>
+    <t>el sistema adapta el contenido</t>
+  </si>
+  <si>
+    <t>Detección de contenido (texto en la página)</t>
+  </si>
+  <si>
+    <t>Activación de la extensión</t>
+  </si>
+  <si>
+    <t>Configuración del usuario (preferencias LSC o Texto)</t>
+  </si>
+  <si>
+    <t>Conversión de texto a LSC</t>
+  </si>
+  <si>
+    <t>Transcripción de audio o video a texto</t>
+  </si>
+  <si>
+    <t>Conversión de audio o video a LSC</t>
+  </si>
+  <si>
+    <t>Confirmaciones accesibles</t>
+  </si>
+  <si>
+    <t>Alertas visuales para eventos importantes</t>
+  </si>
+  <si>
+    <t>Pendiente</t>
+  </si>
+  <si>
+    <t>Parcialmente elaborado</t>
+  </si>
+  <si>
+    <t>Casi listo</t>
+  </si>
+  <si>
+    <t>Listo</t>
   </si>
 </sst>
 </file>
@@ -794,12 +761,26 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -873,8 +854,22 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -939,6 +934,30 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE5CD"/>
         <bgColor rgb="FFFCE5CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1137,15 +1156,15 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1155,8 +1174,8 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1167,26 +1186,14 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1194,116 +1201,125 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="16" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="16" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="16" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="16" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="16" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="16" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1315,11 +1331,50 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1327,7 +1382,85 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{DA6477B6-98E1-4081-AC24-10CDFD97DC67}"/>
     <cellStyle name="Normal 3" xfId="2" xr:uid="{A98AC713-1F17-495A-BFD3-4E6B305F2144}"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="11">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1338,42 +1471,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp1.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp2.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp3.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp4.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp5.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp6.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp7.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp8.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
-</file>
-
-<file path=xl/ctrlProps/ctrlProp9.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1893,614 +1990,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>281940</xdr:colOff>
-          <xdr:row>9</xdr:row>
-          <xdr:rowOff>121920</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>601980</xdr:colOff>
-          <xdr:row>9</xdr:row>
-          <xdr:rowOff>411480</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="2049" name="Check Box 1" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s2049"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000001080000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-                  </a:solidFill>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>266700</xdr:colOff>
-          <xdr:row>8</xdr:row>
-          <xdr:rowOff>106680</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>586740</xdr:colOff>
-          <xdr:row>8</xdr:row>
-          <xdr:rowOff>403860</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="2051" name="Check Box 3" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s2051"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000003080000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-                  </a:solidFill>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>259080</xdr:colOff>
-          <xdr:row>7</xdr:row>
-          <xdr:rowOff>114300</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>579120</xdr:colOff>
-          <xdr:row>7</xdr:row>
-          <xdr:rowOff>403860</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="2055" name="Check Box 7" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s2055"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-000007080000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-                  </a:solidFill>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>281940</xdr:colOff>
-          <xdr:row>10</xdr:row>
-          <xdr:rowOff>121920</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>601980</xdr:colOff>
-          <xdr:row>10</xdr:row>
-          <xdr:rowOff>411480</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="2058" name="Check Box 10" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s2058"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00000A080000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-                  </a:solidFill>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>281940</xdr:colOff>
-          <xdr:row>11</xdr:row>
-          <xdr:rowOff>121920</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>601980</xdr:colOff>
-          <xdr:row>11</xdr:row>
-          <xdr:rowOff>411480</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="2059" name="Check Box 11" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s2059"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00000B080000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-                  </a:solidFill>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>281940</xdr:colOff>
-          <xdr:row>12</xdr:row>
-          <xdr:rowOff>121920</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>601980</xdr:colOff>
-          <xdr:row>12</xdr:row>
-          <xdr:rowOff>411480</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="2060" name="Check Box 12" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s2060"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00000C080000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-                  </a:solidFill>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>281940</xdr:colOff>
-          <xdr:row>13</xdr:row>
-          <xdr:rowOff>121920</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>601980</xdr:colOff>
-          <xdr:row>13</xdr:row>
-          <xdr:rowOff>411480</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="2061" name="Check Box 13" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s2061"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00000D080000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-                  </a:solidFill>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>281940</xdr:colOff>
-          <xdr:row>14</xdr:row>
-          <xdr:rowOff>121920</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>601980</xdr:colOff>
-          <xdr:row>14</xdr:row>
-          <xdr:rowOff>411480</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="2062" name="Check Box 14" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s2062"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00000E080000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-                  </a:solidFill>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
-      <xdr:twoCellAnchor editAs="oneCell">
-        <xdr:from>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>281940</xdr:colOff>
-          <xdr:row>15</xdr:row>
-          <xdr:rowOff>121920</xdr:rowOff>
-        </xdr:from>
-        <xdr:to>
-          <xdr:col>1</xdr:col>
-          <xdr:colOff>601980</xdr:colOff>
-          <xdr:row>16</xdr:row>
-          <xdr:rowOff>159810</xdr:rowOff>
-        </xdr:to>
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="2063" name="Check Box 15" hidden="1">
-              <a:extLst>
-                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s2063"/>
-                </a:ext>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0300-00000F080000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr/>
-          </xdr:nvSpPr>
-          <xdr:spPr bwMode="auto">
-            <a:xfrm>
-              <a:off x="0" y="0"/>
-              <a:ext cx="0" cy="0"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:extLst>
-              <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-                <a14:hiddenFill>
-                  <a:solidFill>
-                    <a:srgbClr val="FFFFFF" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="65"/>
-                  </a:solidFill>
-                </a14:hiddenFill>
-              </a:ext>
-              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-                <a14:hiddenLine w="9525">
-                  <a:solidFill>
-                    <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
-                  </a:solidFill>
-                  <a:miter lim="800000"/>
-                  <a:headEnd/>
-                  <a:tailEnd/>
-                </a14:hiddenLine>
-              </a:ext>
-            </a:extLst>
-          </xdr:spPr>
-        </xdr:sp>
-        <xdr:clientData/>
-      </xdr:twoCellAnchor>
-    </mc:Choice>
-    <mc:Fallback/>
-  </mc:AlternateContent>
-</xdr:wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
@@ -2791,302 +2280,302 @@
   <dimension ref="B1:H30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="2" width="11.5546875" style="21"/>
-    <col min="3" max="3" width="14.44140625" style="21" customWidth="1"/>
-    <col min="4" max="4" width="46.21875" style="21" customWidth="1"/>
-    <col min="5" max="16384" width="11.5546875" style="21"/>
+    <col min="1" max="2" width="11.5546875" style="17"/>
+    <col min="3" max="3" width="14.44140625" style="17" customWidth="1"/>
+    <col min="4" max="4" width="46.21875" style="17" customWidth="1"/>
+    <col min="5" max="16384" width="11.5546875" style="17"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="40.049999999999997" customHeight="1">
-      <c r="B1" s="64" t="s">
-        <v>243</v>
-      </c>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
+      <c r="B1" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
     </row>
     <row r="2" spans="2:8" ht="40.049999999999997" customHeight="1">
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
     </row>
     <row r="3" spans="2:8" ht="40.049999999999997" customHeight="1">
-      <c r="B3" s="64"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
     </row>
     <row r="4" spans="2:8" ht="36" customHeight="1">
-      <c r="B4" s="33" t="s">
-        <v>121</v>
-      </c>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
+      <c r="B4" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
     </row>
     <row r="6" spans="2:8">
-      <c r="B6" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>123</v>
-      </c>
-      <c r="D6" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
+      <c r="B6" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
     </row>
     <row r="7" spans="2:8" ht="36" customHeight="1">
-      <c r="B7" s="24" t="s">
-        <v>125</v>
-      </c>
-      <c r="C7" s="24" t="s">
-        <v>130</v>
-      </c>
-      <c r="D7" s="24" t="s">
-        <v>135</v>
-      </c>
-      <c r="E7" s="22"/>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="22"/>
+      <c r="B7" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
     </row>
     <row r="8" spans="2:8" ht="36" customHeight="1">
-      <c r="B8" s="24" t="s">
-        <v>126</v>
-      </c>
-      <c r="C8" s="24" t="s">
-        <v>131</v>
-      </c>
-      <c r="D8" s="24" t="s">
-        <v>136</v>
-      </c>
-      <c r="E8" s="22"/>
-      <c r="F8" s="22"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
+      <c r="B8" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
     </row>
     <row r="9" spans="2:8" ht="36" customHeight="1">
-      <c r="B9" s="24" t="s">
-        <v>127</v>
-      </c>
-      <c r="C9" s="24" t="s">
-        <v>132</v>
-      </c>
-      <c r="D9" s="24" t="s">
-        <v>137</v>
-      </c>
-      <c r="E9" s="22"/>
-      <c r="F9" s="22"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
+      <c r="B9" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
     </row>
     <row r="10" spans="2:8" ht="36" customHeight="1">
-      <c r="B10" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="C10" s="24" t="s">
-        <v>133</v>
-      </c>
-      <c r="D10" s="24" t="s">
-        <v>138</v>
-      </c>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
+      <c r="B10" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
     </row>
     <row r="11" spans="2:8" ht="36" customHeight="1">
-      <c r="B11" s="24" t="s">
-        <v>129</v>
-      </c>
-      <c r="C11" s="24" t="s">
-        <v>134</v>
-      </c>
-      <c r="D11" s="24" t="s">
-        <v>139</v>
-      </c>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
+      <c r="B11" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
     </row>
     <row r="12" spans="2:8">
-      <c r="B12" s="22"/>
-      <c r="C12" s="22"/>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="22"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
     </row>
     <row r="13" spans="2:8">
-      <c r="B13" s="22"/>
-      <c r="C13" s="22"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="22"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
     </row>
     <row r="14" spans="2:8">
-      <c r="B14" s="22"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="22"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
     </row>
     <row r="15" spans="2:8">
-      <c r="B15" s="22"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
     </row>
     <row r="16" spans="2:8">
-      <c r="B16" s="22"/>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="22"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
+      <c r="B16" s="18"/>
+      <c r="C16" s="18"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
     </row>
     <row r="17" spans="2:8">
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="22"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
     </row>
     <row r="18" spans="2:8">
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="22"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
+      <c r="D18" s="18"/>
+      <c r="E18" s="18"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
     </row>
     <row r="19" spans="2:8">
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="22"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="22"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="18"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
     </row>
     <row r="20" spans="2:8">
-      <c r="B20" s="22"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="22"/>
+      <c r="B20" s="18"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
     </row>
     <row r="21" spans="2:8">
-      <c r="B21" s="22"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="22"/>
+      <c r="B21" s="18"/>
+      <c r="C21" s="18"/>
+      <c r="D21" s="18"/>
+      <c r="E21" s="18"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="18"/>
+      <c r="H21" s="18"/>
     </row>
     <row r="22" spans="2:8">
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="22"/>
+      <c r="B22" s="18"/>
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+      <c r="E22" s="18"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
     </row>
     <row r="23" spans="2:8">
-      <c r="B23" s="22"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="22"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
     </row>
     <row r="24" spans="2:8">
-      <c r="B24" s="22"/>
-      <c r="C24" s="22"/>
-      <c r="D24" s="22"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="22"/>
+      <c r="B24" s="18"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
     </row>
     <row r="25" spans="2:8">
-      <c r="B25" s="22"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="22"/>
-      <c r="E25" s="22"/>
-      <c r="F25" s="22"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="22"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
     </row>
     <row r="26" spans="2:8">
-      <c r="B26" s="22"/>
-      <c r="C26" s="22"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="22"/>
-      <c r="H26" s="22"/>
+      <c r="B26" s="18"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
     </row>
     <row r="27" spans="2:8">
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18"/>
     </row>
     <row r="28" spans="2:8">
-      <c r="B28" s="22"/>
-      <c r="C28" s="22"/>
-      <c r="D28" s="22"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="22"/>
-      <c r="G28" s="22"/>
-      <c r="H28" s="22"/>
+      <c r="B28" s="18"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="18"/>
+      <c r="H28" s="18"/>
     </row>
     <row r="29" spans="2:8">
-      <c r="B29" s="22"/>
-      <c r="C29" s="22"/>
-      <c r="D29" s="22"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="22"/>
-      <c r="G29" s="22"/>
-      <c r="H29" s="22"/>
+      <c r="B29" s="18"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="18"/>
+      <c r="G29" s="18"/>
+      <c r="H29" s="18"/>
     </row>
     <row r="30" spans="2:8">
-      <c r="B30" s="22"/>
-      <c r="C30" s="22"/>
-      <c r="D30" s="22"/>
-      <c r="E30" s="22"/>
-      <c r="F30" s="22"/>
-      <c r="G30" s="22"/>
-      <c r="H30" s="22"/>
+      <c r="B30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3099,7 +2588,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:J41"/>
+  <dimension ref="B1:J38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="1.44140625" style="1" customWidth="1"/>
@@ -3116,34 +2605,34 @@
     <col min="12" max="16384" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" s="21" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="B1" s="64" t="s">
-        <v>243</v>
-      </c>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-    </row>
-    <row r="2" spans="2:10" s="21" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-    </row>
-    <row r="3" spans="2:10" s="21" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="B3" s="64"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
+    <row r="1" spans="2:10" s="17" customFormat="1" ht="40.049999999999997" customHeight="1">
+      <c r="B1" s="37" t="s">
+        <v>149</v>
+      </c>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+    </row>
+    <row r="2" spans="2:10" s="17" customFormat="1" ht="40.049999999999997" customHeight="1">
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+    </row>
+    <row r="3" spans="2:10" s="17" customFormat="1" ht="40.049999999999997" customHeight="1">
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
     </row>
     <row r="4" spans="2:10" ht="36.6" customHeight="1">
       <c r="B4" s="2" t="s">
@@ -3151,18 +2640,18 @@
       </c>
     </row>
     <row r="7" spans="2:10">
-      <c r="C7" s="37" t="s">
+      <c r="C7" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="37"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37" t="s">
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="H7" s="37"/>
-      <c r="I7" s="37"/>
-      <c r="J7" s="37"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="36"/>
     </row>
     <row r="8" spans="2:10" ht="44.25" customHeight="1">
       <c r="B8" s="4" t="s">
@@ -3194,32 +2683,32 @@
       </c>
     </row>
     <row r="9" spans="2:10" ht="42" customHeight="1">
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="38" t="s">
+      <c r="C9" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="34" t="s">
-        <v>100</v>
-      </c>
-      <c r="E9" s="34" t="s">
-        <v>107</v>
+      <c r="D9" s="63" t="s">
+        <v>150</v>
+      </c>
+      <c r="E9" s="63" t="s">
+        <v>151</v>
       </c>
       <c r="F9" s="5">
         <v>1</v>
       </c>
-      <c r="G9" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>17</v>
+      <c r="G9" s="64" t="s">
+        <v>152</v>
+      </c>
+      <c r="H9" s="64" t="s">
+        <v>153</v>
+      </c>
+      <c r="I9" s="64" t="s">
+        <v>154</v>
+      </c>
+      <c r="J9" s="64" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="10" spans="2:10" ht="42" customHeight="1">
@@ -3230,17 +2719,17 @@
       <c r="F10" s="5">
         <v>2</v>
       </c>
-      <c r="G10" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>21</v>
+      <c r="G10" s="64" t="s">
+        <v>156</v>
+      </c>
+      <c r="H10" s="64" t="s">
+        <v>157</v>
+      </c>
+      <c r="I10" s="64" t="s">
+        <v>158</v>
+      </c>
+      <c r="J10" s="64" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="11" spans="2:10">
@@ -3254,54 +2743,54 @@
       <c r="I11" s="12"/>
       <c r="J11" s="12"/>
     </row>
-    <row r="12" spans="2:10" ht="42" customHeight="1">
-      <c r="B12" s="38" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" s="34" t="s">
-        <v>101</v>
-      </c>
-      <c r="D12" s="34" t="s">
-        <v>106</v>
-      </c>
-      <c r="E12" s="34" t="s">
+    <row r="12" spans="2:10" ht="60" customHeight="1">
+      <c r="B12" s="63" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="32" t="s">
         <v>105</v>
+      </c>
+      <c r="D12" s="63" t="s">
+        <v>160</v>
+      </c>
+      <c r="E12" s="63" t="s">
+        <v>161</v>
       </c>
       <c r="F12" s="5">
         <v>1</v>
       </c>
-      <c r="G12" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="2:10" ht="91.2" customHeight="1">
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="35"/>
+      <c r="G12" s="64" t="s">
+        <v>162</v>
+      </c>
+      <c r="H12" s="64" t="s">
+        <v>163</v>
+      </c>
+      <c r="I12" s="65" t="s">
+        <v>164</v>
+      </c>
+      <c r="J12" s="64" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" ht="42" customHeight="1">
+      <c r="B13" s="33"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="33"/>
+      <c r="E13" s="33"/>
       <c r="F13" s="5">
         <v>2</v>
       </c>
-      <c r="G13" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="J13" s="6" t="s">
-        <v>30</v>
+      <c r="G13" s="16" t="s">
+        <v>106</v>
+      </c>
+      <c r="H13" s="64" t="s">
+        <v>166</v>
+      </c>
+      <c r="I13" s="64" t="s">
+        <v>167</v>
+      </c>
+      <c r="J13" s="64" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="14" spans="2:10">
@@ -3316,53 +2805,53 @@
       <c r="J14" s="12"/>
     </row>
     <row r="15" spans="2:10" ht="42" customHeight="1">
-      <c r="B15" s="38" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="D15" s="34" t="s">
-        <v>108</v>
-      </c>
-      <c r="E15" s="34" t="s">
-        <v>109</v>
+      <c r="B15" s="63" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="63" t="s">
+        <v>169</v>
+      </c>
+      <c r="D15" s="63" t="s">
+        <v>170</v>
+      </c>
+      <c r="E15" s="63" t="s">
+        <v>171</v>
       </c>
       <c r="F15" s="5">
         <v>1</v>
       </c>
-      <c r="G15" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="I15" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="J15" s="6" t="s">
-        <v>35</v>
+      <c r="G15" s="64" t="s">
+        <v>172</v>
+      </c>
+      <c r="H15" s="64" t="s">
+        <v>173</v>
+      </c>
+      <c r="I15" s="65" t="s">
+        <v>164</v>
+      </c>
+      <c r="J15" s="64" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="16" spans="2:10" ht="42" customHeight="1">
-      <c r="B16" s="36"/>
-      <c r="C16" s="36"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="36"/>
+      <c r="B16" s="33"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
       <c r="F16" s="5">
         <v>2</v>
       </c>
-      <c r="G16" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="J16" s="6" t="s">
-        <v>39</v>
+      <c r="G16" s="64" t="s">
+        <v>175</v>
+      </c>
+      <c r="H16" s="64" t="s">
+        <v>176</v>
+      </c>
+      <c r="I16" s="64" t="s">
+        <v>177</v>
+      </c>
+      <c r="J16" s="64" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="17" spans="2:10">
@@ -3377,53 +2866,53 @@
       <c r="J17" s="12"/>
     </row>
     <row r="18" spans="2:10" ht="42" customHeight="1">
-      <c r="B18" s="34" t="s">
-        <v>103</v>
-      </c>
-      <c r="C18" s="38" t="s">
+      <c r="B18" s="63" t="s">
+        <v>79</v>
+      </c>
+      <c r="C18" s="34" t="s">
         <v>13</v>
       </c>
-      <c r="D18" s="34" t="s">
-        <v>104</v>
-      </c>
-      <c r="E18" s="34" t="s">
-        <v>110</v>
+      <c r="D18" s="63" t="s">
+        <v>181</v>
+      </c>
+      <c r="E18" s="63" t="s">
+        <v>182</v>
       </c>
       <c r="F18" s="5">
         <v>1</v>
       </c>
-      <c r="G18" s="19" t="s">
-        <v>18</v>
-      </c>
-      <c r="H18" s="19" t="s">
-        <v>113</v>
-      </c>
-      <c r="I18" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="J18" s="19" t="s">
-        <v>112</v>
+      <c r="G18" s="64" t="s">
+        <v>183</v>
+      </c>
+      <c r="H18" s="64" t="s">
+        <v>184</v>
+      </c>
+      <c r="I18" s="65" t="s">
+        <v>185</v>
+      </c>
+      <c r="J18" s="64" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="19" spans="2:10" ht="42" customHeight="1">
-      <c r="B19" s="36"/>
-      <c r="C19" s="36"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="36"/>
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
       <c r="F19" s="5">
         <v>2</v>
       </c>
-      <c r="G19" s="19" t="s">
-        <v>114</v>
-      </c>
-      <c r="H19" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="I19" s="19" t="s">
-        <v>116</v>
-      </c>
-      <c r="J19" s="19" t="s">
-        <v>117</v>
+      <c r="G19" s="64" t="s">
+        <v>187</v>
+      </c>
+      <c r="H19" s="64" t="s">
+        <v>188</v>
+      </c>
+      <c r="I19" s="64" t="s">
+        <v>189</v>
+      </c>
+      <c r="J19" s="64" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="20" spans="2:10">
@@ -3437,54 +2926,54 @@
       <c r="I20" s="12"/>
       <c r="J20" s="12"/>
     </row>
-    <row r="21" spans="2:10" ht="66" customHeight="1">
-      <c r="B21" s="34" t="s">
-        <v>140</v>
+    <row r="21" spans="2:10" ht="42" customHeight="1">
+      <c r="B21" s="63" t="s">
+        <v>101</v>
       </c>
       <c r="C21" s="34" t="s">
-        <v>145</v>
-      </c>
-      <c r="D21" s="34" t="s">
-        <v>146</v>
-      </c>
-      <c r="E21" s="34" t="s">
-        <v>147</v>
+        <v>13</v>
+      </c>
+      <c r="D21" s="63" t="s">
+        <v>191</v>
+      </c>
+      <c r="E21" s="63" t="s">
+        <v>192</v>
       </c>
       <c r="F21" s="5">
         <v>1</v>
       </c>
-      <c r="G21" s="19" t="s">
-        <v>151</v>
-      </c>
-      <c r="H21" s="19" t="s">
-        <v>148</v>
-      </c>
-      <c r="I21" s="25" t="s">
-        <v>149</v>
-      </c>
-      <c r="J21" s="19" t="s">
-        <v>150</v>
+      <c r="G21" s="64" t="s">
+        <v>193</v>
+      </c>
+      <c r="H21" s="64" t="s">
+        <v>194</v>
+      </c>
+      <c r="I21" s="65" t="s">
+        <v>195</v>
+      </c>
+      <c r="J21" s="64" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="22" spans="2:10" ht="42" customHeight="1">
-      <c r="B22" s="36"/>
-      <c r="C22" s="36"/>
-      <c r="D22" s="36"/>
-      <c r="E22" s="36"/>
+      <c r="B22" s="33"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="33"/>
+      <c r="E22" s="33"/>
       <c r="F22" s="5">
         <v>2</v>
       </c>
-      <c r="G22" s="19" t="s">
-        <v>152</v>
-      </c>
-      <c r="H22" s="19" t="s">
-        <v>153</v>
-      </c>
-      <c r="I22" s="19" t="s">
-        <v>154</v>
-      </c>
-      <c r="J22" s="19" t="s">
-        <v>155</v>
+      <c r="G22" s="64" t="s">
+        <v>197</v>
+      </c>
+      <c r="H22" s="64" t="s">
+        <v>198</v>
+      </c>
+      <c r="I22" s="64" t="s">
+        <v>199</v>
+      </c>
+      <c r="J22" s="64" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="23" spans="2:10">
@@ -3498,54 +2987,54 @@
       <c r="I23" s="12"/>
       <c r="J23" s="12"/>
     </row>
-    <row r="24" spans="2:10" ht="60" customHeight="1">
-      <c r="B24" s="34" t="s">
-        <v>141</v>
+    <row r="24" spans="2:10" ht="42" customHeight="1">
+      <c r="B24" s="63" t="s">
+        <v>102</v>
       </c>
       <c r="C24" s="34" t="s">
-        <v>145</v>
-      </c>
-      <c r="D24" s="34" t="s">
-        <v>156</v>
-      </c>
-      <c r="E24" s="34" t="s">
-        <v>157</v>
+        <v>13</v>
+      </c>
+      <c r="D24" s="63" t="s">
+        <v>201</v>
+      </c>
+      <c r="E24" s="63" t="s">
+        <v>179</v>
       </c>
       <c r="F24" s="5">
         <v>1</v>
       </c>
-      <c r="G24" s="19" t="s">
-        <v>158</v>
-      </c>
-      <c r="H24" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="I24" s="20" t="s">
-        <v>160</v>
-      </c>
-      <c r="J24" s="19" t="s">
-        <v>161</v>
+      <c r="G24" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="H24" s="64" t="s">
+        <v>202</v>
+      </c>
+      <c r="I24" s="65" t="s">
+        <v>203</v>
+      </c>
+      <c r="J24" s="64" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="25" spans="2:10" ht="42" customHeight="1">
-      <c r="B25" s="36"/>
-      <c r="C25" s="36"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="36"/>
+      <c r="B25" s="33"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
       <c r="F25" s="5">
         <v>2</v>
       </c>
-      <c r="G25" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="H25" s="19" t="s">
-        <v>163</v>
-      </c>
-      <c r="I25" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="J25" s="19" t="s">
-        <v>165</v>
+      <c r="G25" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H25" s="64" t="s">
+        <v>205</v>
+      </c>
+      <c r="I25" s="64" t="s">
+        <v>180</v>
+      </c>
+      <c r="J25" s="64" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="26" spans="2:10">
@@ -3560,53 +3049,53 @@
       <c r="J26" s="12"/>
     </row>
     <row r="27" spans="2:10" ht="42" customHeight="1">
-      <c r="B27" s="34" t="s">
-        <v>142</v>
-      </c>
-      <c r="C27" s="34" t="s">
+      <c r="B27" s="63" t="s">
+        <v>103</v>
+      </c>
+      <c r="C27" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="D27" s="34" t="s">
-        <v>166</v>
-      </c>
-      <c r="E27" s="34" t="s">
-        <v>167</v>
+      <c r="D27" s="63" t="s">
+        <v>107</v>
+      </c>
+      <c r="E27" s="63" t="s">
+        <v>206</v>
       </c>
       <c r="F27" s="5">
         <v>1</v>
       </c>
-      <c r="G27" s="19" t="s">
-        <v>168</v>
-      </c>
-      <c r="H27" s="19" t="s">
-        <v>169</v>
-      </c>
-      <c r="I27" s="20" t="s">
-        <v>170</v>
-      </c>
-      <c r="J27" s="19" t="s">
-        <v>171</v>
+      <c r="G27" s="16" t="s">
+        <v>108</v>
+      </c>
+      <c r="H27" s="64" t="s">
+        <v>207</v>
+      </c>
+      <c r="I27" s="65" t="s">
+        <v>208</v>
+      </c>
+      <c r="J27" s="16" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="28" spans="2:10" ht="42" customHeight="1">
-      <c r="B28" s="36"/>
-      <c r="C28" s="36"/>
-      <c r="D28" s="36"/>
-      <c r="E28" s="36"/>
+      <c r="B28" s="33"/>
+      <c r="C28" s="33"/>
+      <c r="D28" s="33"/>
+      <c r="E28" s="33"/>
       <c r="F28" s="5">
         <v>2</v>
       </c>
-      <c r="G28" s="19" t="s">
-        <v>172</v>
-      </c>
-      <c r="H28" s="19" t="s">
-        <v>173</v>
-      </c>
-      <c r="I28" s="19" t="s">
-        <v>174</v>
-      </c>
-      <c r="J28" s="19" t="s">
-        <v>175</v>
+      <c r="G28" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="H28" s="64" t="s">
+        <v>209</v>
+      </c>
+      <c r="I28" s="64" t="s">
+        <v>111</v>
+      </c>
+      <c r="J28" s="64" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="29" spans="2:10">
@@ -3621,53 +3110,53 @@
       <c r="J29" s="12"/>
     </row>
     <row r="30" spans="2:10" ht="42" customHeight="1">
-      <c r="B30" s="34" t="s">
-        <v>143</v>
-      </c>
-      <c r="C30" s="34" t="s">
-        <v>176</v>
-      </c>
-      <c r="D30" s="34" t="s">
-        <v>177</v>
-      </c>
-      <c r="E30" s="34" t="s">
-        <v>178</v>
+      <c r="B30" s="63" t="s">
+        <v>104</v>
+      </c>
+      <c r="C30" s="32" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" s="63" t="s">
+        <v>211</v>
+      </c>
+      <c r="E30" s="63" t="s">
+        <v>212</v>
       </c>
       <c r="F30" s="5">
         <v>1</v>
       </c>
-      <c r="G30" s="19" t="s">
-        <v>179</v>
-      </c>
-      <c r="H30" s="19" t="s">
-        <v>180</v>
-      </c>
-      <c r="I30" s="20" t="s">
-        <v>181</v>
-      </c>
-      <c r="J30" s="19" t="s">
-        <v>182</v>
+      <c r="G30" s="64" t="s">
+        <v>213</v>
+      </c>
+      <c r="H30" s="64" t="s">
+        <v>215</v>
+      </c>
+      <c r="I30" s="65" t="s">
+        <v>216</v>
+      </c>
+      <c r="J30" s="64" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="31" spans="2:10" ht="42" customHeight="1">
-      <c r="B31" s="36"/>
-      <c r="C31" s="36"/>
-      <c r="D31" s="36"/>
-      <c r="E31" s="36"/>
+      <c r="B31" s="33"/>
+      <c r="C31" s="33"/>
+      <c r="D31" s="33"/>
+      <c r="E31" s="33"/>
       <c r="F31" s="5">
         <v>2</v>
       </c>
-      <c r="G31" s="19" t="s">
-        <v>183</v>
-      </c>
-      <c r="H31" s="19" t="s">
-        <v>184</v>
-      </c>
-      <c r="I31" s="19" t="s">
-        <v>185</v>
-      </c>
-      <c r="J31" s="19" t="s">
-        <v>186</v>
+      <c r="G31" s="64" t="s">
+        <v>214</v>
+      </c>
+      <c r="H31" s="64" t="s">
+        <v>218</v>
+      </c>
+      <c r="I31" s="64" t="s">
+        <v>219</v>
+      </c>
+      <c r="J31" s="64" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="32" spans="2:10">
@@ -3681,118 +3170,52 @@
       <c r="I32" s="12"/>
       <c r="J32" s="12"/>
     </row>
-    <row r="33" spans="2:10" ht="42" customHeight="1">
-      <c r="B33" s="34" t="s">
-        <v>144</v>
-      </c>
-      <c r="C33" s="34" t="s">
-        <v>13</v>
-      </c>
-      <c r="D33" s="34" t="s">
-        <v>201</v>
-      </c>
-      <c r="E33" s="34" t="s">
-        <v>187</v>
-      </c>
-      <c r="F33" s="5">
-        <v>1</v>
-      </c>
-      <c r="G33" s="19" t="s">
-        <v>188</v>
-      </c>
-      <c r="H33" s="19" t="s">
-        <v>189</v>
-      </c>
-      <c r="I33" s="20" t="s">
-        <v>190</v>
-      </c>
-      <c r="J33" s="19" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="34" spans="2:10" ht="42" customHeight="1">
-      <c r="B34" s="36"/>
-      <c r="C34" s="36"/>
-      <c r="D34" s="36"/>
-      <c r="E34" s="36"/>
-      <c r="F34" s="5">
-        <v>2</v>
-      </c>
-      <c r="G34" s="19" t="s">
-        <v>192</v>
-      </c>
-      <c r="H34" s="19" t="s">
-        <v>193</v>
-      </c>
-      <c r="I34" s="19" t="s">
-        <v>194</v>
-      </c>
-      <c r="J34" s="19" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="35" spans="2:10">
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="11"/>
-      <c r="G35" s="12"/>
-      <c r="H35" s="12"/>
-      <c r="I35" s="12"/>
-      <c r="J35" s="12"/>
-    </row>
-    <row r="37" spans="2:10">
-      <c r="B37" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="38" spans="2:10">
-      <c r="B38" s="13" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="39" spans="2:10">
-      <c r="B39" s="13" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="41" spans="2:10" ht="21">
-      <c r="B41" s="3" t="s">
-        <v>43</v>
+    <row r="34" spans="2:2">
+      <c r="B34" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2">
+      <c r="B35" s="13" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2">
+      <c r="B36" s="13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2" ht="21">
+      <c r="B38" s="3" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="39">
-    <mergeCell ref="B1:H3"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="E24:E25"/>
+  <mergeCells count="35">
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="E18:E19"/>
     <mergeCell ref="B21:B22"/>
     <mergeCell ref="C21:C22"/>
     <mergeCell ref="D21:D22"/>
     <mergeCell ref="E21:E22"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B1:H3"/>
     <mergeCell ref="G7:J7"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:E25"/>
     <mergeCell ref="C7:F7"/>
     <mergeCell ref="B9:B10"/>
     <mergeCell ref="C9:C10"/>
     <mergeCell ref="D9:D10"/>
     <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="C33:C34"/>
-    <mergeCell ref="D33:D34"/>
-    <mergeCell ref="E33:E34"/>
     <mergeCell ref="B30:B31"/>
     <mergeCell ref="C30:C31"/>
     <mergeCell ref="D30:D31"/>
@@ -3801,8 +3224,9 @@
     <mergeCell ref="C27:C28"/>
     <mergeCell ref="D27:D28"/>
     <mergeCell ref="E27:E28"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="70" orientation="landscape"/>
@@ -3819,178 +3243,178 @@
     <col min="7" max="16384" width="11.5546875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" s="21" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="B1" s="64" t="s">
-        <v>243</v>
-      </c>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-    </row>
-    <row r="2" spans="2:10" s="21" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="64"/>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
-    </row>
-    <row r="3" spans="2:10" s="21" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="B3" s="64"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="64"/>
-      <c r="I3" s="64"/>
-      <c r="J3" s="64"/>
+    <row r="1" spans="2:10" s="17" customFormat="1" ht="40.049999999999997" customHeight="1">
+      <c r="B1" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+    </row>
+    <row r="2" spans="2:10" s="17" customFormat="1" ht="40.049999999999997" customHeight="1">
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="J2" s="31"/>
+    </row>
+    <row r="3" spans="2:10" s="17" customFormat="1" ht="40.049999999999997" customHeight="1">
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
     </row>
     <row r="4" spans="2:10" ht="36" customHeight="1">
       <c r="C4" s="2" t="s">
-        <v>120</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="2:10">
-      <c r="C6" s="50" t="s">
-        <v>72</v>
-      </c>
-      <c r="D6" s="50"/>
-      <c r="E6" s="50"/>
-      <c r="G6" s="51" t="s">
-        <v>73</v>
-      </c>
-      <c r="H6" s="51"/>
-      <c r="I6" s="51"/>
+      <c r="C6" s="49" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="49"/>
+      <c r="E6" s="49"/>
+      <c r="G6" s="50" t="s">
+        <v>52</v>
+      </c>
+      <c r="H6" s="50"/>
+      <c r="I6" s="50"/>
     </row>
     <row r="7" spans="2:10">
-      <c r="C7" s="45" t="s">
-        <v>74</v>
-      </c>
-      <c r="D7" s="46"/>
-      <c r="E7" s="47"/>
-      <c r="G7" s="45" t="s">
-        <v>75</v>
-      </c>
-      <c r="H7" s="46"/>
-      <c r="I7" s="47"/>
+      <c r="C7" s="44" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="45"/>
+      <c r="E7" s="46"/>
+      <c r="G7" s="44" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" s="45"/>
+      <c r="I7" s="46"/>
     </row>
     <row r="8" spans="2:10">
-      <c r="C8" s="39" t="s">
-        <v>76</v>
-      </c>
-      <c r="D8" s="40"/>
-      <c r="E8" s="41"/>
-      <c r="G8" s="39" t="s">
-        <v>77</v>
-      </c>
-      <c r="H8" s="40"/>
-      <c r="I8" s="41"/>
+      <c r="C8" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="39"/>
+      <c r="E8" s="40"/>
+      <c r="G8" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="H8" s="39"/>
+      <c r="I8" s="40"/>
     </row>
     <row r="9" spans="2:10">
-      <c r="C9" s="39" t="s">
-        <v>78</v>
-      </c>
-      <c r="D9" s="40"/>
-      <c r="E9" s="41"/>
-      <c r="G9" s="39" t="s">
-        <v>79</v>
-      </c>
-      <c r="H9" s="40"/>
-      <c r="I9" s="41"/>
+      <c r="C9" s="38" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="39"/>
+      <c r="E9" s="40"/>
+      <c r="G9" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="H9" s="39"/>
+      <c r="I9" s="40"/>
     </row>
     <row r="10" spans="2:10">
-      <c r="C10" s="39"/>
-      <c r="D10" s="40"/>
-      <c r="E10" s="41"/>
-      <c r="G10" s="52" t="s">
-        <v>80</v>
-      </c>
-      <c r="H10" s="53"/>
-      <c r="I10" s="54"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="39"/>
+      <c r="E10" s="40"/>
+      <c r="G10" s="51" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" s="52"/>
+      <c r="I10" s="53"/>
     </row>
     <row r="11" spans="2:10">
-      <c r="C11" s="42"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="44"/>
-      <c r="G11" s="55"/>
-      <c r="H11" s="56"/>
-      <c r="I11" s="57"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="43"/>
+      <c r="G11" s="54"/>
+      <c r="H11" s="55"/>
+      <c r="I11" s="56"/>
     </row>
     <row r="12" spans="2:10" ht="9" customHeight="1"/>
     <row r="13" spans="2:10">
-      <c r="C13" s="48" t="s">
-        <v>81</v>
-      </c>
-      <c r="D13" s="48"/>
-      <c r="E13" s="48"/>
-      <c r="G13" s="49" t="s">
-        <v>82</v>
-      </c>
-      <c r="H13" s="49"/>
-      <c r="I13" s="49"/>
+      <c r="C13" s="47" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="47"/>
+      <c r="E13" s="47"/>
+      <c r="G13" s="48" t="s">
+        <v>61</v>
+      </c>
+      <c r="H13" s="48"/>
+      <c r="I13" s="48"/>
     </row>
     <row r="14" spans="2:10">
-      <c r="C14" s="45" t="s">
-        <v>83</v>
-      </c>
-      <c r="D14" s="46"/>
-      <c r="E14" s="47"/>
-      <c r="G14" s="45" t="s">
-        <v>84</v>
-      </c>
-      <c r="H14" s="46"/>
-      <c r="I14" s="47"/>
+      <c r="C14" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="D14" s="45"/>
+      <c r="E14" s="46"/>
+      <c r="G14" s="44" t="s">
+        <v>63</v>
+      </c>
+      <c r="H14" s="45"/>
+      <c r="I14" s="46"/>
     </row>
     <row r="15" spans="2:10">
-      <c r="C15" s="39" t="s">
-        <v>85</v>
-      </c>
-      <c r="D15" s="40"/>
-      <c r="E15" s="41"/>
-      <c r="G15" s="39" t="s">
-        <v>86</v>
-      </c>
-      <c r="H15" s="40"/>
-      <c r="I15" s="41"/>
+      <c r="C15" s="38" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="39"/>
+      <c r="E15" s="40"/>
+      <c r="G15" s="38" t="s">
+        <v>65</v>
+      </c>
+      <c r="H15" s="39"/>
+      <c r="I15" s="40"/>
     </row>
     <row r="16" spans="2:10">
-      <c r="C16" s="39" t="s">
-        <v>87</v>
-      </c>
-      <c r="D16" s="40"/>
-      <c r="E16" s="41"/>
-      <c r="G16" s="39" t="s">
-        <v>88</v>
-      </c>
-      <c r="H16" s="40"/>
-      <c r="I16" s="41"/>
+      <c r="C16" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="D16" s="39"/>
+      <c r="E16" s="40"/>
+      <c r="G16" s="38" t="s">
+        <v>67</v>
+      </c>
+      <c r="H16" s="39"/>
+      <c r="I16" s="40"/>
     </row>
     <row r="17" spans="3:9">
-      <c r="C17" s="39"/>
-      <c r="D17" s="40"/>
-      <c r="E17" s="41"/>
-      <c r="G17" s="39" t="s">
-        <v>89</v>
-      </c>
-      <c r="H17" s="40"/>
-      <c r="I17" s="41"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="39"/>
+      <c r="E17" s="40"/>
+      <c r="G17" s="38" t="s">
+        <v>68</v>
+      </c>
+      <c r="H17" s="39"/>
+      <c r="I17" s="40"/>
     </row>
     <row r="18" spans="3:9">
-      <c r="C18" s="42"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="44"/>
-      <c r="G18" s="42"/>
-      <c r="H18" s="43"/>
-      <c r="I18" s="44"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="42"/>
+      <c r="E18" s="43"/>
+      <c r="G18" s="41"/>
+      <c r="H18" s="42"/>
+      <c r="I18" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="24">
@@ -4025,8 +3449,8 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D425717-E79E-458E-BEB7-0CA397B048CB}">
-  <dimension ref="A1:I17"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D425717-E79E-458E-BEB7-0CA397B048CB}">
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="3" width="11.5546875" style="14"/>
@@ -4035,425 +3459,296 @@
     <col min="6" max="16384" width="11.5546875" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="14.4" customHeight="1">
-      <c r="A1" s="65"/>
-      <c r="B1" s="65"/>
-      <c r="C1" s="65"/>
-      <c r="D1" s="65"/>
-      <c r="E1" s="65"/>
-      <c r="F1" s="65"/>
-      <c r="G1" s="65"/>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-    </row>
-    <row r="2" spans="1:9" ht="40.049999999999997" customHeight="1">
-      <c r="A2" s="65"/>
-      <c r="B2" s="64" t="s">
-        <v>243</v>
-      </c>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-    </row>
-    <row r="3" spans="1:9" ht="40.049999999999997" customHeight="1">
-      <c r="A3" s="65"/>
-      <c r="B3" s="64"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
-      <c r="H3" s="65"/>
-      <c r="I3" s="65"/>
-    </row>
-    <row r="4" spans="1:9" ht="40.049999999999997" customHeight="1">
-      <c r="B4" s="64"/>
-      <c r="C4" s="64"/>
-      <c r="D4" s="64"/>
-      <c r="E4" s="64"/>
-      <c r="F4" s="64"/>
-      <c r="G4" s="64"/>
-    </row>
-    <row r="5" spans="1:9" ht="36" customHeight="1"/>
-    <row r="6" spans="1:9" ht="36" customHeight="1">
-      <c r="B6" s="58" t="s">
-        <v>90</v>
-      </c>
-      <c r="C6" s="59"/>
-      <c r="D6" s="59"/>
-      <c r="E6" s="59"/>
-      <c r="F6" s="60"/>
-    </row>
-    <row r="7" spans="1:9" ht="36" customHeight="1">
+    <row r="1" spans="1:10" ht="14.4" customHeight="1">
+      <c r="A1" s="28"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+    </row>
+    <row r="2" spans="1:10" ht="40.049999999999997" customHeight="1">
+      <c r="A2" s="28"/>
+      <c r="B2" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+    </row>
+    <row r="3" spans="1:10" ht="40.049999999999997" customHeight="1">
+      <c r="A3" s="28"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="28"/>
+      <c r="I3" s="28"/>
+    </row>
+    <row r="4" spans="1:10" ht="40.049999999999997" customHeight="1">
+      <c r="B4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="31"/>
+    </row>
+    <row r="5" spans="1:10" ht="36" customHeight="1"/>
+    <row r="6" spans="1:10" ht="36" customHeight="1">
+      <c r="B6" s="57" t="s">
+        <v>69</v>
+      </c>
+      <c r="C6" s="58"/>
+      <c r="D6" s="58"/>
+      <c r="E6" s="58"/>
+      <c r="F6" s="59"/>
+    </row>
+    <row r="7" spans="1:10" ht="36" customHeight="1">
       <c r="B7" s="15" t="s">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>92</v>
+        <v>71</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>94</v>
+        <v>73</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="36" customHeight="1">
-      <c r="B8" s="15"/>
-      <c r="C8" s="15" t="s">
-        <v>96</v>
-      </c>
-      <c r="D8" s="18" t="s">
-        <v>202</v>
-      </c>
-      <c r="E8" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="F8" s="15">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" s="29" customFormat="1" ht="21.6" customHeight="1">
+      <c r="B8" s="66" t="s">
+        <v>129</v>
+      </c>
+      <c r="C8" s="67"/>
+      <c r="D8" s="67"/>
+      <c r="E8" s="67"/>
+      <c r="F8" s="68"/>
+      <c r="H8" s="73"/>
+      <c r="I8" s="77" t="s">
+        <v>229</v>
+      </c>
+      <c r="J8" s="39"/>
+    </row>
+    <row r="9" spans="1:10" ht="36" customHeight="1">
+      <c r="B9" s="72">
+        <v>2</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="69" t="s">
+        <v>221</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="F9" s="15">
         <v>3</v>
       </c>
-    </row>
-    <row r="9" spans="1:9" ht="36" customHeight="1">
-      <c r="B9" s="15"/>
-      <c r="C9" s="15" t="s">
-        <v>97</v>
-      </c>
-      <c r="D9" s="18" t="s">
-        <v>203</v>
-      </c>
-      <c r="E9" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="F9" s="15">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="36" customHeight="1">
-      <c r="B10" s="15"/>
-      <c r="C10" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="D10" s="18" t="s">
-        <v>102</v>
+      <c r="H9" s="74"/>
+      <c r="I9" s="77" t="s">
+        <v>230</v>
+      </c>
+      <c r="J9" s="39"/>
+    </row>
+    <row r="10" spans="1:10" ht="36" customHeight="1">
+      <c r="B10" s="72">
+        <v>3</v>
+      </c>
+      <c r="C10" s="70" t="s">
+        <v>112</v>
+      </c>
+      <c r="D10" s="69" t="s">
+        <v>222</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>99</v>
+        <v>78</v>
       </c>
       <c r="F10" s="15">
+        <v>2</v>
+      </c>
+      <c r="H10" s="75"/>
+      <c r="I10" s="77" t="s">
+        <v>231</v>
+      </c>
+      <c r="J10" s="39"/>
+    </row>
+    <row r="11" spans="1:10" ht="36" customHeight="1">
+      <c r="B11" s="72">
+        <v>2</v>
+      </c>
+      <c r="C11" s="70" t="s">
+        <v>115</v>
+      </c>
+      <c r="D11" s="69" t="s">
+        <v>223</v>
+      </c>
+      <c r="E11" s="70" t="s">
+        <v>78</v>
+      </c>
+      <c r="F11" s="15">
+        <v>3</v>
+      </c>
+      <c r="H11" s="76"/>
+      <c r="I11" s="77" t="s">
+        <v>232</v>
+      </c>
+      <c r="J11" s="39"/>
+    </row>
+    <row r="12" spans="1:10" s="29" customFormat="1" ht="21.6" customHeight="1">
+      <c r="B12" s="66" t="s">
+        <v>133</v>
+      </c>
+      <c r="C12" s="67"/>
+      <c r="D12" s="67"/>
+      <c r="E12" s="67"/>
+      <c r="F12" s="68"/>
+    </row>
+    <row r="13" spans="1:10" ht="36" customHeight="1">
+      <c r="B13" s="72">
+        <v>2</v>
+      </c>
+      <c r="C13" s="70" t="s">
+        <v>76</v>
+      </c>
+      <c r="D13" s="70" t="s">
+        <v>224</v>
+      </c>
+      <c r="E13" s="70" t="s">
+        <v>78</v>
+      </c>
+      <c r="F13" s="15">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="36" customHeight="1">
-      <c r="B11" s="15"/>
-      <c r="C11" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>119</v>
-      </c>
-      <c r="E11" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="F11" s="15">
+    <row r="14" spans="1:10" ht="36" customHeight="1">
+      <c r="B14" s="72">
+        <v>1</v>
+      </c>
+      <c r="C14" s="70" t="s">
+        <v>77</v>
+      </c>
+      <c r="D14" s="70" t="s">
+        <v>225</v>
+      </c>
+      <c r="E14" s="70" t="s">
+        <v>78</v>
+      </c>
+      <c r="F14" s="15">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="36" customHeight="1">
-      <c r="B12" s="15"/>
-      <c r="C12" s="15" t="s">
-        <v>196</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>204</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="F12" s="15">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="36" customHeight="1">
-      <c r="B13" s="15"/>
-      <c r="C13" s="15" t="s">
-        <v>197</v>
-      </c>
-      <c r="D13" s="18" t="s">
-        <v>205</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>99</v>
-      </c>
-      <c r="F13" s="15">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" ht="36" customHeight="1">
-      <c r="B14" s="15"/>
-      <c r="C14" s="15" t="s">
-        <v>198</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>210</v>
-      </c>
-      <c r="E14" s="17" t="s">
-        <v>209</v>
-      </c>
-      <c r="F14" s="15">
+    <row r="15" spans="1:10" s="29" customFormat="1" ht="21.6" customHeight="1">
+      <c r="B15" s="66" t="s">
+        <v>136</v>
+      </c>
+      <c r="C15" s="67"/>
+      <c r="D15" s="67"/>
+      <c r="E15" s="67"/>
+      <c r="F15" s="68"/>
+    </row>
+    <row r="16" spans="1:10" ht="36" customHeight="1">
+      <c r="B16" s="72">
+        <v>1</v>
+      </c>
+      <c r="C16" s="70" t="s">
+        <v>80</v>
+      </c>
+      <c r="D16" s="70" t="s">
+        <v>226</v>
+      </c>
+      <c r="E16" s="70" t="s">
+        <v>116</v>
+      </c>
+      <c r="F16" s="15">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" ht="36" customHeight="1">
+      <c r="B17" s="72">
+        <v>1</v>
+      </c>
+      <c r="C17" s="70" t="s">
+        <v>113</v>
+      </c>
+      <c r="D17" s="70" t="s">
+        <v>227</v>
+      </c>
+      <c r="E17" s="70" t="s">
+        <v>116</v>
+      </c>
+      <c r="F17" s="15">
+        <v>3</v>
+      </c>
+      <c r="H17" s="71"/>
+    </row>
+    <row r="18" spans="2:8" ht="36" customHeight="1">
+      <c r="B18" s="72">
+        <v>1</v>
+      </c>
+      <c r="C18" s="70" t="s">
+        <v>114</v>
+      </c>
+      <c r="D18" s="70" t="s">
+        <v>228</v>
+      </c>
+      <c r="E18" s="70" t="s">
+        <v>116</v>
+      </c>
+      <c r="F18" s="15">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="36" customHeight="1">
-      <c r="B15" s="15"/>
-      <c r="C15" s="15" t="s">
-        <v>199</v>
-      </c>
-      <c r="D15" s="18" t="s">
-        <v>206</v>
-      </c>
-      <c r="E15" s="17" t="s">
-        <v>208</v>
-      </c>
-      <c r="F15" s="15">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" ht="19.95" customHeight="1">
-      <c r="B16" s="15"/>
-      <c r="C16" s="15" t="s">
-        <v>200</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>207</v>
-      </c>
-      <c r="E16" s="17" t="s">
-        <v>208</v>
-      </c>
-      <c r="F16" s="15">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" ht="19.95" customHeight="1"/>
+    <row r="19" spans="2:8" ht="19.95" customHeight="1">
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+    </row>
+    <row r="20" spans="2:8" ht="19.95" customHeight="1"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="9">
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="I9:J9"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="I11:J11"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B2:G4"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B15:F15"/>
   </mergeCells>
-  <phoneticPr fontId="9" type="noConversion"/>
+  <phoneticPr fontId="11" type="noConversion"/>
+  <conditionalFormatting sqref="B9:B11 B13:B14 B16:B18">
+    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
+      <formula>1</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+      <formula>2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+      <formula>3</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+      <formula>4</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x14">
-      <controls>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="2049" r:id="rId3" name="Check Box 1">
-              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>281940</xdr:colOff>
-                    <xdr:row>9</xdr:row>
-                    <xdr:rowOff>121920</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>601980</xdr:colOff>
-                    <xdr:row>9</xdr:row>
-                    <xdr:rowOff>411480</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="2051" r:id="rId4" name="Check Box 3">
-              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>266700</xdr:colOff>
-                    <xdr:row>8</xdr:row>
-                    <xdr:rowOff>106680</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>586740</xdr:colOff>
-                    <xdr:row>8</xdr:row>
-                    <xdr:rowOff>403860</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="2055" r:id="rId5" name="Check Box 7">
-              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>259080</xdr:colOff>
-                    <xdr:row>7</xdr:row>
-                    <xdr:rowOff>114300</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>579120</xdr:colOff>
-                    <xdr:row>7</xdr:row>
-                    <xdr:rowOff>403860</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="2058" r:id="rId6" name="Check Box 10">
-              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>281940</xdr:colOff>
-                    <xdr:row>10</xdr:row>
-                    <xdr:rowOff>121920</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>601980</xdr:colOff>
-                    <xdr:row>10</xdr:row>
-                    <xdr:rowOff>411480</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="2059" r:id="rId7" name="Check Box 11">
-              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>281940</xdr:colOff>
-                    <xdr:row>11</xdr:row>
-                    <xdr:rowOff>121920</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>601980</xdr:colOff>
-                    <xdr:row>11</xdr:row>
-                    <xdr:rowOff>411480</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="2060" r:id="rId8" name="Check Box 12">
-              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>281940</xdr:colOff>
-                    <xdr:row>12</xdr:row>
-                    <xdr:rowOff>121920</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>601980</xdr:colOff>
-                    <xdr:row>12</xdr:row>
-                    <xdr:rowOff>411480</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="2061" r:id="rId9" name="Check Box 13">
-              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>281940</xdr:colOff>
-                    <xdr:row>13</xdr:row>
-                    <xdr:rowOff>121920</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>601980</xdr:colOff>
-                    <xdr:row>13</xdr:row>
-                    <xdr:rowOff>411480</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="2062" r:id="rId10" name="Check Box 14">
-              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>281940</xdr:colOff>
-                    <xdr:row>14</xdr:row>
-                    <xdr:rowOff>121920</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>601980</xdr:colOff>
-                    <xdr:row>14</xdr:row>
-                    <xdr:rowOff>411480</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-        <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-          <mc:Choice Requires="x14">
-            <control shapeId="2063" r:id="rId11" name="Check Box 15">
-              <controlPr defaultSize="0" autoFill="0" autoLine="0" autoPict="0">
-                <anchor moveWithCells="1">
-                  <from>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>281940</xdr:colOff>
-                    <xdr:row>15</xdr:row>
-                    <xdr:rowOff>121920</xdr:rowOff>
-                  </from>
-                  <to>
-                    <xdr:col>1</xdr:col>
-                    <xdr:colOff>601980</xdr:colOff>
-                    <xdr:row>16</xdr:row>
-                    <xdr:rowOff>160020</xdr:rowOff>
-                  </to>
-                </anchor>
-              </controlPr>
-            </control>
-          </mc:Choice>
-        </mc:AlternateContent>
-      </controls>
-    </mc:Choice>
-  </mc:AlternateContent>
 </worksheet>
 </file>
 
@@ -4462,224 +3757,224 @@
   <dimension ref="A1:I1003"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="20" style="29" customWidth="1"/>
-    <col min="2" max="2" width="21.109375" style="29" customWidth="1"/>
-    <col min="3" max="3" width="29.6640625" style="29" customWidth="1"/>
-    <col min="4" max="6" width="15.88671875" style="29" customWidth="1"/>
-    <col min="7" max="26" width="8.6640625" style="29" customWidth="1"/>
-    <col min="27" max="16384" width="14.44140625" style="29"/>
+    <col min="1" max="1" width="20" style="24" customWidth="1"/>
+    <col min="2" max="2" width="21.109375" style="24" customWidth="1"/>
+    <col min="3" max="3" width="29.6640625" style="24" customWidth="1"/>
+    <col min="4" max="6" width="15.88671875" style="24" customWidth="1"/>
+    <col min="7" max="26" width="8.6640625" style="24" customWidth="1"/>
+    <col min="27" max="16384" width="14.44140625" style="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="26" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="A1" s="65"/>
-      <c r="B1" s="64" t="s">
-        <v>243</v>
-      </c>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="65"/>
-      <c r="I1" s="65"/>
-    </row>
-    <row r="2" spans="1:9" s="26" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="A2" s="65"/>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="64"/>
-      <c r="F2" s="64"/>
-      <c r="G2" s="64"/>
-      <c r="H2" s="65"/>
-      <c r="I2" s="65"/>
-    </row>
-    <row r="3" spans="1:9" s="26" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="B3" s="64"/>
-      <c r="C3" s="64"/>
-      <c r="D3" s="64"/>
-      <c r="E3" s="64"/>
-      <c r="F3" s="64"/>
-      <c r="G3" s="64"/>
+    <row r="1" spans="1:9" s="21" customFormat="1" ht="40.049999999999997" customHeight="1">
+      <c r="A1" s="28"/>
+      <c r="B1" s="31" t="s">
+        <v>149</v>
+      </c>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="28"/>
+      <c r="I1" s="28"/>
+    </row>
+    <row r="2" spans="1:9" s="21" customFormat="1" ht="40.049999999999997" customHeight="1">
+      <c r="A2" s="28"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="28"/>
+      <c r="I2" s="28"/>
+    </row>
+    <row r="3" spans="1:9" s="21" customFormat="1" ht="40.049999999999997" customHeight="1">
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
     </row>
     <row r="4" spans="1:9" ht="28.8">
-      <c r="A4" s="27" t="s">
-        <v>211</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>212</v>
-      </c>
-      <c r="C4" s="28" t="s">
+      <c r="A4" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="B4" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>85</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>119</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="F4" s="23" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="28.8">
+      <c r="A5" s="25" t="s">
+        <v>122</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>123</v>
+      </c>
+      <c r="C5" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="D4" s="28" t="s">
-        <v>213</v>
-      </c>
-      <c r="E4" s="28" t="s">
-        <v>214</v>
-      </c>
-      <c r="F4" s="28" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" ht="28.8">
-      <c r="A5" s="30" t="s">
-        <v>216</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>217</v>
-      </c>
-      <c r="C5" s="31" t="s">
-        <v>218</v>
-      </c>
-      <c r="D5" s="32">
+      <c r="D5" s="27">
         <v>46065</v>
       </c>
-      <c r="E5" s="32">
+      <c r="E5" s="27">
         <v>46071</v>
       </c>
-      <c r="F5" s="31" t="s">
-        <v>219</v>
+      <c r="F5" s="26" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="28.8">
-      <c r="A6" s="30" t="s">
-        <v>220</v>
-      </c>
-      <c r="B6" s="31" t="s">
-        <v>221</v>
-      </c>
-      <c r="C6" s="31" t="s">
-        <v>222</v>
-      </c>
-      <c r="D6" s="32">
+      <c r="A6" s="25" t="s">
+        <v>126</v>
+      </c>
+      <c r="B6" s="26" t="s">
+        <v>127</v>
+      </c>
+      <c r="C6" s="26" t="s">
+        <v>128</v>
+      </c>
+      <c r="D6" s="27">
         <v>46072</v>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="27">
         <v>46078</v>
       </c>
-      <c r="F6" s="31" t="s">
-        <v>219</v>
+      <c r="F6" s="26" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="43.2">
-      <c r="A7" s="30" t="s">
-        <v>223</v>
-      </c>
-      <c r="B7" s="31" t="s">
-        <v>224</v>
-      </c>
-      <c r="C7" s="31" t="s">
-        <v>225</v>
-      </c>
-      <c r="D7" s="32">
+      <c r="A7" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="B7" s="26" t="s">
+        <v>130</v>
+      </c>
+      <c r="C7" s="26" t="s">
+        <v>131</v>
+      </c>
+      <c r="D7" s="27">
         <v>46079</v>
       </c>
-      <c r="E7" s="32">
+      <c r="E7" s="27">
         <v>46092</v>
       </c>
-      <c r="F7" s="31" t="s">
-        <v>226</v>
+      <c r="F7" s="26" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="28.8">
-      <c r="A8" s="30" t="s">
-        <v>227</v>
-      </c>
-      <c r="B8" s="31" t="s">
-        <v>228</v>
-      </c>
-      <c r="C8" s="31" t="s">
-        <v>229</v>
-      </c>
-      <c r="D8" s="32">
+      <c r="A8" s="25" t="s">
+        <v>133</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>134</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>135</v>
+      </c>
+      <c r="D8" s="27">
         <v>46093</v>
       </c>
-      <c r="E8" s="32">
+      <c r="E8" s="27">
         <v>46106</v>
       </c>
-      <c r="F8" s="31" t="s">
-        <v>226</v>
+      <c r="F8" s="26" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="28.8">
-      <c r="A9" s="30" t="s">
-        <v>230</v>
-      </c>
-      <c r="B9" s="31" t="s">
-        <v>231</v>
-      </c>
-      <c r="C9" s="31" t="s">
-        <v>232</v>
-      </c>
-      <c r="D9" s="32">
+      <c r="A9" s="25" t="s">
+        <v>136</v>
+      </c>
+      <c r="B9" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>138</v>
+      </c>
+      <c r="D9" s="27">
         <v>46107</v>
       </c>
-      <c r="E9" s="32">
+      <c r="E9" s="27">
         <v>46120</v>
       </c>
-      <c r="F9" s="31" t="s">
-        <v>226</v>
+      <c r="F9" s="26" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="43.2">
-      <c r="A10" s="30" t="s">
-        <v>233</v>
-      </c>
-      <c r="B10" s="31" t="s">
-        <v>234</v>
-      </c>
-      <c r="C10" s="31" t="s">
-        <v>235</v>
-      </c>
-      <c r="D10" s="32">
+      <c r="A10" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10" s="26" t="s">
+        <v>140</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="D10" s="27">
         <v>46121</v>
       </c>
-      <c r="E10" s="32">
+      <c r="E10" s="27">
         <v>46134</v>
       </c>
-      <c r="F10" s="31" t="s">
-        <v>226</v>
+      <c r="F10" s="26" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="28.8">
-      <c r="A11" s="30" t="s">
-        <v>236</v>
-      </c>
-      <c r="B11" s="31" t="s">
-        <v>237</v>
-      </c>
-      <c r="C11" s="31" t="s">
-        <v>238</v>
-      </c>
-      <c r="D11" s="32">
+      <c r="A11" s="25" t="s">
+        <v>142</v>
+      </c>
+      <c r="B11" s="26" t="s">
+        <v>143</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>144</v>
+      </c>
+      <c r="D11" s="27">
         <v>46135</v>
       </c>
-      <c r="E11" s="32">
+      <c r="E11" s="27">
         <v>46155</v>
       </c>
-      <c r="F11" s="31" t="s">
-        <v>239</v>
+      <c r="F11" s="26" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="28.8">
-      <c r="A12" s="30" t="s">
-        <v>240</v>
-      </c>
-      <c r="B12" s="31" t="s">
-        <v>241</v>
-      </c>
-      <c r="C12" s="31" t="s">
-        <v>242</v>
-      </c>
-      <c r="D12" s="32">
+      <c r="A12" s="25" t="s">
+        <v>146</v>
+      </c>
+      <c r="B12" s="26" t="s">
+        <v>147</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>148</v>
+      </c>
+      <c r="D12" s="27">
         <v>46156</v>
       </c>
-      <c r="E12" s="32">
+      <c r="E12" s="27">
         <v>46178</v>
       </c>
-      <c r="F12" s="31" t="s">
-        <v>239</v>
+      <c r="F12" s="26" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1"/>
@@ -5685,20 +4980,20 @@
   <sheetData>
     <row r="1" spans="2:3" ht="31.2">
       <c r="B1" s="8" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="2:3" ht="21">
       <c r="B2" s="3" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="2:3">
       <c r="B4" s="9" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="2:3" ht="28.8">
@@ -5706,7 +5001,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="2:3" ht="129.6">
@@ -5714,7 +5009,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="2:3" ht="100.8">
@@ -5722,7 +5017,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>49</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="2:3" ht="43.2">
@@ -5730,7 +5025,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>50</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="2:3">
@@ -5738,15 +5033,15 @@
         <v>7</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>51</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="2:3" ht="43.2">
       <c r="B10" s="6" t="s">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>53</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="2:3">
@@ -5754,7 +5049,7 @@
         <v>9</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>54</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="2:3">
@@ -5762,7 +5057,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>55</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="2:3" ht="28.8">
@@ -5770,7 +5065,7 @@
         <v>11</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>56</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -5800,27 +5095,27 @@
   <sheetData>
     <row r="1" spans="2:10" ht="36.6">
       <c r="B1" s="2" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="2:10" ht="21">
       <c r="B2" s="3" t="s">
-        <v>43</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="2:10">
-      <c r="C4" s="37" t="s">
+      <c r="C4" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="37"/>
-      <c r="E4" s="37"/>
-      <c r="F4" s="37"/>
-      <c r="G4" s="37" t="s">
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="H4" s="37"/>
-      <c r="I4" s="37"/>
-      <c r="J4" s="37"/>
+      <c r="H4" s="36"/>
+      <c r="I4" s="36"/>
+      <c r="J4" s="36"/>
     </row>
     <row r="5" spans="2:10" ht="28.8">
       <c r="B5" s="4" t="s">
@@ -5852,81 +5147,81 @@
       </c>
     </row>
     <row r="6" spans="2:10" ht="57.6">
-      <c r="B6" s="61" t="s">
-        <v>58</v>
-      </c>
-      <c r="C6" s="61" t="s">
-        <v>59</v>
-      </c>
-      <c r="D6" s="61" t="s">
-        <v>60</v>
-      </c>
-      <c r="E6" s="61" t="s">
-        <v>61</v>
+      <c r="B6" s="60" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="60" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="60" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="60" t="s">
+        <v>40</v>
       </c>
       <c r="F6" s="5">
         <v>1</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>65</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="2:10" ht="72">
-      <c r="B7" s="62"/>
-      <c r="C7" s="62"/>
-      <c r="D7" s="62"/>
-      <c r="E7" s="62"/>
+      <c r="B7" s="61"/>
+      <c r="C7" s="61"/>
+      <c r="D7" s="61"/>
+      <c r="E7" s="61"/>
       <c r="F7" s="5">
         <v>2</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>66</v>
+        <v>45</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="2:10" ht="43.2">
-      <c r="B8" s="62"/>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
+      <c r="B8" s="61"/>
+      <c r="C8" s="61"/>
+      <c r="D8" s="61"/>
+      <c r="E8" s="61"/>
       <c r="F8" s="5">
         <v>3</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>69</v>
+        <v>48</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>70</v>
+        <v>49</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>71</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="2:10">
-      <c r="B9" s="63"/>
-      <c r="C9" s="63"/>
-      <c r="D9" s="63"/>
-      <c r="E9" s="63"/>
+      <c r="B9" s="62"/>
+      <c r="C9" s="62"/>
+      <c r="D9" s="62"/>
+      <c r="E9" s="62"/>
       <c r="F9" s="5"/>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>

</xml_diff>

<commit_message>
Cambios Santiago: ajustar configuración del usuario
</commit_message>
<xml_diff>
--- a/Docs/Proyecto.xlsx
+++ b/Docs/Proyecto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PERSONAL\Desktop\Universidad\Sexto semestre 2026 - I\Ingeneria de software II\AsistenteVirtual\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E2FDE4A-B034-4469-A741-9B53DDAD7AC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE32C7B2-A368-439A-8831-CBAB98D30976}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1232,29 +1232,83 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1265,6 +1319,24 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1274,44 +1346,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1322,6 +1358,15 @@
     <xf numFmtId="0" fontId="9" fillId="3" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1330,51 +1375,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1382,28 +1382,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{DA6477B6-98E1-4081-AC24-10CDFD97DC67}"/>
     <cellStyle name="Normal 3" xfId="2" xr:uid="{A98AC713-1F17-495A-BFD3-4E6B305F2144}"/>
   </cellStyles>
-  <dxfs count="11">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill>
@@ -1422,34 +1401,6 @@
       <fill>
         <patternFill>
           <bgColor theme="9" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="-0.24994659260841701"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2287,34 +2238,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="40.049999999999997" customHeight="1">
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="41" t="s">
         <v>149</v>
       </c>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
     </row>
     <row r="2" spans="2:8" ht="40.049999999999997" customHeight="1">
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
     </row>
     <row r="3" spans="2:8" ht="40.049999999999997" customHeight="1">
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
     </row>
     <row r="4" spans="2:8" ht="36" customHeight="1">
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="40" t="s">
         <v>82</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
     </row>
     <row r="6" spans="2:8">
       <c r="B6" s="19" t="s">
@@ -2606,33 +2557,33 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" s="17" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="B1" s="37" t="s">
+      <c r="B1" s="46" t="s">
         <v>149</v>
       </c>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
     </row>
     <row r="2" spans="2:10" s="17" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="2:10" s="17" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
     </row>
     <row r="4" spans="2:10" ht="36.6" customHeight="1">
       <c r="B4" s="2" t="s">
@@ -2640,18 +2591,18 @@
       </c>
     </row>
     <row r="7" spans="2:10">
-      <c r="C7" s="36" t="s">
+      <c r="C7" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="G7" s="36" t="s">
+      <c r="D7" s="47"/>
+      <c r="E7" s="47"/>
+      <c r="F7" s="47"/>
+      <c r="G7" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="H7" s="36"/>
-      <c r="I7" s="36"/>
-      <c r="J7" s="36"/>
+      <c r="H7" s="47"/>
+      <c r="I7" s="47"/>
+      <c r="J7" s="47"/>
     </row>
     <row r="8" spans="2:10" ht="44.25" customHeight="1">
       <c r="B8" s="4" t="s">
@@ -2683,52 +2634,52 @@
       </c>
     </row>
     <row r="9" spans="2:10" ht="42" customHeight="1">
-      <c r="B9" s="34" t="s">
+      <c r="B9" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="63" t="s">
+      <c r="D9" s="42" t="s">
         <v>150</v>
       </c>
-      <c r="E9" s="63" t="s">
+      <c r="E9" s="42" t="s">
         <v>151</v>
       </c>
       <c r="F9" s="5">
         <v>1</v>
       </c>
-      <c r="G9" s="64" t="s">
+      <c r="G9" s="30" t="s">
         <v>152</v>
       </c>
-      <c r="H9" s="64" t="s">
+      <c r="H9" s="30" t="s">
         <v>153</v>
       </c>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="30" t="s">
         <v>154</v>
       </c>
-      <c r="J9" s="64" t="s">
+      <c r="J9" s="30" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="10" spans="2:10" ht="42" customHeight="1">
-      <c r="B10" s="35"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="35"/>
+      <c r="B10" s="48"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
       <c r="F10" s="5">
         <v>2</v>
       </c>
-      <c r="G10" s="64" t="s">
+      <c r="G10" s="30" t="s">
         <v>156</v>
       </c>
-      <c r="H10" s="64" t="s">
+      <c r="H10" s="30" t="s">
         <v>157</v>
       </c>
-      <c r="I10" s="64" t="s">
+      <c r="I10" s="30" t="s">
         <v>158</v>
       </c>
-      <c r="J10" s="64" t="s">
+      <c r="J10" s="30" t="s">
         <v>159</v>
       </c>
     </row>
@@ -2744,52 +2695,52 @@
       <c r="J11" s="12"/>
     </row>
     <row r="12" spans="2:10" ht="60" customHeight="1">
-      <c r="B12" s="63" t="s">
+      <c r="B12" s="42" t="s">
         <v>14</v>
       </c>
-      <c r="C12" s="32" t="s">
+      <c r="C12" s="44" t="s">
         <v>105</v>
       </c>
-      <c r="D12" s="63" t="s">
+      <c r="D12" s="42" t="s">
         <v>160</v>
       </c>
-      <c r="E12" s="63" t="s">
+      <c r="E12" s="42" t="s">
         <v>161</v>
       </c>
       <c r="F12" s="5">
         <v>1</v>
       </c>
-      <c r="G12" s="64" t="s">
+      <c r="G12" s="30" t="s">
         <v>162</v>
       </c>
-      <c r="H12" s="64" t="s">
+      <c r="H12" s="30" t="s">
         <v>163</v>
       </c>
-      <c r="I12" s="65" t="s">
+      <c r="I12" s="31" t="s">
         <v>164</v>
       </c>
-      <c r="J12" s="64" t="s">
+      <c r="J12" s="30" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="13" spans="2:10" ht="42" customHeight="1">
-      <c r="B13" s="33"/>
-      <c r="C13" s="33"/>
-      <c r="D13" s="33"/>
-      <c r="E13" s="33"/>
+      <c r="B13" s="43"/>
+      <c r="C13" s="43"/>
+      <c r="D13" s="43"/>
+      <c r="E13" s="43"/>
       <c r="F13" s="5">
         <v>2</v>
       </c>
       <c r="G13" s="16" t="s">
         <v>106</v>
       </c>
-      <c r="H13" s="64" t="s">
+      <c r="H13" s="30" t="s">
         <v>166</v>
       </c>
-      <c r="I13" s="64" t="s">
+      <c r="I13" s="30" t="s">
         <v>167</v>
       </c>
-      <c r="J13" s="64" t="s">
+      <c r="J13" s="30" t="s">
         <v>168</v>
       </c>
     </row>
@@ -2805,52 +2756,52 @@
       <c r="J14" s="12"/>
     </row>
     <row r="15" spans="2:10" ht="42" customHeight="1">
-      <c r="B15" s="63" t="s">
+      <c r="B15" s="42" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="63" t="s">
+      <c r="C15" s="42" t="s">
         <v>169</v>
       </c>
-      <c r="D15" s="63" t="s">
+      <c r="D15" s="42" t="s">
         <v>170</v>
       </c>
-      <c r="E15" s="63" t="s">
+      <c r="E15" s="42" t="s">
         <v>171</v>
       </c>
       <c r="F15" s="5">
         <v>1</v>
       </c>
-      <c r="G15" s="64" t="s">
+      <c r="G15" s="30" t="s">
         <v>172</v>
       </c>
-      <c r="H15" s="64" t="s">
+      <c r="H15" s="30" t="s">
         <v>173</v>
       </c>
-      <c r="I15" s="65" t="s">
+      <c r="I15" s="31" t="s">
         <v>164</v>
       </c>
-      <c r="J15" s="64" t="s">
+      <c r="J15" s="30" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="16" spans="2:10" ht="42" customHeight="1">
-      <c r="B16" s="33"/>
-      <c r="C16" s="33"/>
-      <c r="D16" s="33"/>
-      <c r="E16" s="33"/>
+      <c r="B16" s="43"/>
+      <c r="C16" s="43"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="43"/>
       <c r="F16" s="5">
         <v>2</v>
       </c>
-      <c r="G16" s="64" t="s">
+      <c r="G16" s="30" t="s">
         <v>175</v>
       </c>
-      <c r="H16" s="64" t="s">
+      <c r="H16" s="30" t="s">
         <v>176</v>
       </c>
-      <c r="I16" s="64" t="s">
+      <c r="I16" s="30" t="s">
         <v>177</v>
       </c>
-      <c r="J16" s="64" t="s">
+      <c r="J16" s="30" t="s">
         <v>178</v>
       </c>
     </row>
@@ -2866,52 +2817,52 @@
       <c r="J17" s="12"/>
     </row>
     <row r="18" spans="2:10" ht="42" customHeight="1">
-      <c r="B18" s="63" t="s">
+      <c r="B18" s="42" t="s">
         <v>79</v>
       </c>
-      <c r="C18" s="34" t="s">
+      <c r="C18" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="D18" s="63" t="s">
+      <c r="D18" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="E18" s="63" t="s">
+      <c r="E18" s="42" t="s">
         <v>182</v>
       </c>
       <c r="F18" s="5">
         <v>1</v>
       </c>
-      <c r="G18" s="64" t="s">
+      <c r="G18" s="30" t="s">
         <v>183</v>
       </c>
-      <c r="H18" s="64" t="s">
+      <c r="H18" s="30" t="s">
         <v>184</v>
       </c>
-      <c r="I18" s="65" t="s">
+      <c r="I18" s="31" t="s">
         <v>185</v>
       </c>
-      <c r="J18" s="64" t="s">
+      <c r="J18" s="30" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="19" spans="2:10" ht="42" customHeight="1">
-      <c r="B19" s="33"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="33"/>
-      <c r="E19" s="33"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="43"/>
       <c r="F19" s="5">
         <v>2</v>
       </c>
-      <c r="G19" s="64" t="s">
+      <c r="G19" s="30" t="s">
         <v>187</v>
       </c>
-      <c r="H19" s="64" t="s">
+      <c r="H19" s="30" t="s">
         <v>188</v>
       </c>
-      <c r="I19" s="64" t="s">
+      <c r="I19" s="30" t="s">
         <v>189</v>
       </c>
-      <c r="J19" s="64" t="s">
+      <c r="J19" s="30" t="s">
         <v>190</v>
       </c>
     </row>
@@ -2927,52 +2878,52 @@
       <c r="J20" s="12"/>
     </row>
     <row r="21" spans="2:10" ht="42" customHeight="1">
-      <c r="B21" s="63" t="s">
+      <c r="B21" s="42" t="s">
         <v>101</v>
       </c>
-      <c r="C21" s="34" t="s">
+      <c r="C21" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="D21" s="63" t="s">
+      <c r="D21" s="42" t="s">
         <v>191</v>
       </c>
-      <c r="E21" s="63" t="s">
+      <c r="E21" s="42" t="s">
         <v>192</v>
       </c>
       <c r="F21" s="5">
         <v>1</v>
       </c>
-      <c r="G21" s="64" t="s">
+      <c r="G21" s="30" t="s">
         <v>193</v>
       </c>
-      <c r="H21" s="64" t="s">
+      <c r="H21" s="30" t="s">
         <v>194</v>
       </c>
-      <c r="I21" s="65" t="s">
+      <c r="I21" s="31" t="s">
         <v>195</v>
       </c>
-      <c r="J21" s="64" t="s">
+      <c r="J21" s="30" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="22" spans="2:10" ht="42" customHeight="1">
-      <c r="B22" s="33"/>
-      <c r="C22" s="33"/>
-      <c r="D22" s="33"/>
-      <c r="E22" s="33"/>
+      <c r="B22" s="43"/>
+      <c r="C22" s="43"/>
+      <c r="D22" s="43"/>
+      <c r="E22" s="43"/>
       <c r="F22" s="5">
         <v>2</v>
       </c>
-      <c r="G22" s="64" t="s">
+      <c r="G22" s="30" t="s">
         <v>197</v>
       </c>
-      <c r="H22" s="64" t="s">
+      <c r="H22" s="30" t="s">
         <v>198</v>
       </c>
-      <c r="I22" s="64" t="s">
+      <c r="I22" s="30" t="s">
         <v>199</v>
       </c>
-      <c r="J22" s="64" t="s">
+      <c r="J22" s="30" t="s">
         <v>200</v>
       </c>
     </row>
@@ -2988,16 +2939,16 @@
       <c r="J23" s="12"/>
     </row>
     <row r="24" spans="2:10" ht="42" customHeight="1">
-      <c r="B24" s="63" t="s">
+      <c r="B24" s="42" t="s">
         <v>102</v>
       </c>
-      <c r="C24" s="34" t="s">
+      <c r="C24" s="45" t="s">
         <v>13</v>
       </c>
-      <c r="D24" s="63" t="s">
+      <c r="D24" s="42" t="s">
         <v>201</v>
       </c>
-      <c r="E24" s="63" t="s">
+      <c r="E24" s="42" t="s">
         <v>179</v>
       </c>
       <c r="F24" s="5">
@@ -3006,34 +2957,34 @@
       <c r="G24" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="H24" s="64" t="s">
+      <c r="H24" s="30" t="s">
         <v>202</v>
       </c>
-      <c r="I24" s="65" t="s">
+      <c r="I24" s="31" t="s">
         <v>203</v>
       </c>
-      <c r="J24" s="64" t="s">
+      <c r="J24" s="30" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="25" spans="2:10" ht="42" customHeight="1">
-      <c r="B25" s="33"/>
-      <c r="C25" s="33"/>
-      <c r="D25" s="33"/>
-      <c r="E25" s="33"/>
+      <c r="B25" s="43"/>
+      <c r="C25" s="43"/>
+      <c r="D25" s="43"/>
+      <c r="E25" s="43"/>
       <c r="F25" s="5">
         <v>2</v>
       </c>
       <c r="G25" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="H25" s="64" t="s">
+      <c r="H25" s="30" t="s">
         <v>205</v>
       </c>
-      <c r="I25" s="64" t="s">
+      <c r="I25" s="30" t="s">
         <v>180</v>
       </c>
-      <c r="J25" s="64" t="s">
+      <c r="J25" s="30" t="s">
         <v>18</v>
       </c>
     </row>
@@ -3049,16 +3000,16 @@
       <c r="J26" s="12"/>
     </row>
     <row r="27" spans="2:10" ht="42" customHeight="1">
-      <c r="B27" s="63" t="s">
+      <c r="B27" s="42" t="s">
         <v>103</v>
       </c>
-      <c r="C27" s="32" t="s">
+      <c r="C27" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="D27" s="63" t="s">
+      <c r="D27" s="42" t="s">
         <v>107</v>
       </c>
-      <c r="E27" s="63" t="s">
+      <c r="E27" s="42" t="s">
         <v>206</v>
       </c>
       <c r="F27" s="5">
@@ -3067,10 +3018,10 @@
       <c r="G27" s="16" t="s">
         <v>108</v>
       </c>
-      <c r="H27" s="64" t="s">
+      <c r="H27" s="30" t="s">
         <v>207</v>
       </c>
-      <c r="I27" s="65" t="s">
+      <c r="I27" s="31" t="s">
         <v>208</v>
       </c>
       <c r="J27" s="16" t="s">
@@ -3078,23 +3029,23 @@
       </c>
     </row>
     <row r="28" spans="2:10" ht="42" customHeight="1">
-      <c r="B28" s="33"/>
-      <c r="C28" s="33"/>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
+      <c r="B28" s="43"/>
+      <c r="C28" s="43"/>
+      <c r="D28" s="43"/>
+      <c r="E28" s="43"/>
       <c r="F28" s="5">
         <v>2</v>
       </c>
       <c r="G28" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="H28" s="64" t="s">
+      <c r="H28" s="30" t="s">
         <v>209</v>
       </c>
-      <c r="I28" s="64" t="s">
+      <c r="I28" s="30" t="s">
         <v>111</v>
       </c>
-      <c r="J28" s="64" t="s">
+      <c r="J28" s="30" t="s">
         <v>210</v>
       </c>
     </row>
@@ -3110,52 +3061,52 @@
       <c r="J29" s="12"/>
     </row>
     <row r="30" spans="2:10" ht="42" customHeight="1">
-      <c r="B30" s="63" t="s">
+      <c r="B30" s="42" t="s">
         <v>104</v>
       </c>
-      <c r="C30" s="32" t="s">
+      <c r="C30" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="D30" s="63" t="s">
+      <c r="D30" s="42" t="s">
         <v>211</v>
       </c>
-      <c r="E30" s="63" t="s">
+      <c r="E30" s="42" t="s">
         <v>212</v>
       </c>
       <c r="F30" s="5">
         <v>1</v>
       </c>
-      <c r="G30" s="64" t="s">
+      <c r="G30" s="30" t="s">
         <v>213</v>
       </c>
-      <c r="H30" s="64" t="s">
+      <c r="H30" s="30" t="s">
         <v>215</v>
       </c>
-      <c r="I30" s="65" t="s">
+      <c r="I30" s="31" t="s">
         <v>216</v>
       </c>
-      <c r="J30" s="64" t="s">
+      <c r="J30" s="30" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="31" spans="2:10" ht="42" customHeight="1">
-      <c r="B31" s="33"/>
-      <c r="C31" s="33"/>
-      <c r="D31" s="33"/>
-      <c r="E31" s="33"/>
+      <c r="B31" s="43"/>
+      <c r="C31" s="43"/>
+      <c r="D31" s="43"/>
+      <c r="E31" s="43"/>
       <c r="F31" s="5">
         <v>2</v>
       </c>
-      <c r="G31" s="64" t="s">
+      <c r="G31" s="30" t="s">
         <v>214</v>
       </c>
-      <c r="H31" s="64" t="s">
+      <c r="H31" s="30" t="s">
         <v>218</v>
       </c>
-      <c r="I31" s="64" t="s">
+      <c r="I31" s="30" t="s">
         <v>219</v>
       </c>
-      <c r="J31" s="64" t="s">
+      <c r="J31" s="30" t="s">
         <v>220</v>
       </c>
     </row>
@@ -3192,19 +3143,14 @@
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="D12:D13"/>
-    <mergeCell ref="E12:E13"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="E30:E31"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="E27:E28"/>
     <mergeCell ref="B1:H3"/>
     <mergeCell ref="G7:J7"/>
     <mergeCell ref="B24:B25"/>
@@ -3216,17 +3162,22 @@
     <mergeCell ref="C9:C10"/>
     <mergeCell ref="D9:D10"/>
     <mergeCell ref="E9:E10"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="E30:E31"/>
-    <mergeCell ref="B27:B28"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="E27:E28"/>
     <mergeCell ref="B15:B16"/>
     <mergeCell ref="C15:C16"/>
     <mergeCell ref="D15:D16"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="E18:E19"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="70" orientation="landscape"/>
@@ -3244,39 +3195,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:10" s="17" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="41" t="s">
         <v>149</v>
       </c>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
     </row>
     <row r="2" spans="2:10" s="17" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
+      <c r="I2" s="41"/>
+      <c r="J2" s="41"/>
     </row>
     <row r="3" spans="2:10" s="17" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
-      <c r="J3" s="31"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
+      <c r="I3" s="41"/>
+      <c r="J3" s="41"/>
     </row>
     <row r="4" spans="2:10" ht="36" customHeight="1">
       <c r="C4" s="2" t="s">
@@ -3284,140 +3235,150 @@
       </c>
     </row>
     <row r="6" spans="2:10">
-      <c r="C6" s="49" t="s">
+      <c r="C6" s="51" t="s">
         <v>51</v>
       </c>
-      <c r="D6" s="49"/>
-      <c r="E6" s="49"/>
-      <c r="G6" s="50" t="s">
+      <c r="D6" s="51"/>
+      <c r="E6" s="51"/>
+      <c r="G6" s="52" t="s">
         <v>52</v>
       </c>
-      <c r="H6" s="50"/>
-      <c r="I6" s="50"/>
+      <c r="H6" s="52"/>
+      <c r="I6" s="52"/>
     </row>
     <row r="7" spans="2:10">
-      <c r="C7" s="44" t="s">
+      <c r="C7" s="53" t="s">
         <v>53</v>
       </c>
-      <c r="D7" s="45"/>
-      <c r="E7" s="46"/>
-      <c r="G7" s="44" t="s">
+      <c r="D7" s="54"/>
+      <c r="E7" s="55"/>
+      <c r="G7" s="53" t="s">
         <v>54</v>
       </c>
-      <c r="H7" s="45"/>
-      <c r="I7" s="46"/>
+      <c r="H7" s="54"/>
+      <c r="I7" s="55"/>
     </row>
     <row r="8" spans="2:10">
-      <c r="C8" s="38" t="s">
+      <c r="C8" s="56" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="39"/>
-      <c r="E8" s="40"/>
-      <c r="G8" s="38" t="s">
+      <c r="D8" s="57"/>
+      <c r="E8" s="58"/>
+      <c r="G8" s="56" t="s">
         <v>56</v>
       </c>
-      <c r="H8" s="39"/>
-      <c r="I8" s="40"/>
+      <c r="H8" s="57"/>
+      <c r="I8" s="58"/>
     </row>
     <row r="9" spans="2:10">
-      <c r="C9" s="38" t="s">
+      <c r="C9" s="56" t="s">
         <v>57</v>
       </c>
-      <c r="D9" s="39"/>
-      <c r="E9" s="40"/>
-      <c r="G9" s="38" t="s">
+      <c r="D9" s="57"/>
+      <c r="E9" s="58"/>
+      <c r="G9" s="56" t="s">
         <v>58</v>
       </c>
-      <c r="H9" s="39"/>
-      <c r="I9" s="40"/>
+      <c r="H9" s="57"/>
+      <c r="I9" s="58"/>
     </row>
     <row r="10" spans="2:10">
-      <c r="C10" s="38"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="40"/>
-      <c r="G10" s="51" t="s">
+      <c r="C10" s="56"/>
+      <c r="D10" s="57"/>
+      <c r="E10" s="58"/>
+      <c r="G10" s="59" t="s">
         <v>59</v>
       </c>
-      <c r="H10" s="52"/>
-      <c r="I10" s="53"/>
+      <c r="H10" s="60"/>
+      <c r="I10" s="61"/>
     </row>
     <row r="11" spans="2:10">
-      <c r="C11" s="41"/>
-      <c r="D11" s="42"/>
-      <c r="E11" s="43"/>
-      <c r="G11" s="54"/>
-      <c r="H11" s="55"/>
-      <c r="I11" s="56"/>
+      <c r="C11" s="65"/>
+      <c r="D11" s="66"/>
+      <c r="E11" s="67"/>
+      <c r="G11" s="62"/>
+      <c r="H11" s="63"/>
+      <c r="I11" s="64"/>
     </row>
     <row r="12" spans="2:10" ht="9" customHeight="1"/>
     <row r="13" spans="2:10">
-      <c r="C13" s="47" t="s">
+      <c r="C13" s="49" t="s">
         <v>60</v>
       </c>
-      <c r="D13" s="47"/>
-      <c r="E13" s="47"/>
-      <c r="G13" s="48" t="s">
+      <c r="D13" s="49"/>
+      <c r="E13" s="49"/>
+      <c r="G13" s="50" t="s">
         <v>61</v>
       </c>
-      <c r="H13" s="48"/>
-      <c r="I13" s="48"/>
+      <c r="H13" s="50"/>
+      <c r="I13" s="50"/>
     </row>
     <row r="14" spans="2:10">
-      <c r="C14" s="44" t="s">
+      <c r="C14" s="53" t="s">
         <v>62</v>
       </c>
-      <c r="D14" s="45"/>
-      <c r="E14" s="46"/>
-      <c r="G14" s="44" t="s">
+      <c r="D14" s="54"/>
+      <c r="E14" s="55"/>
+      <c r="G14" s="53" t="s">
         <v>63</v>
       </c>
-      <c r="H14" s="45"/>
-      <c r="I14" s="46"/>
+      <c r="H14" s="54"/>
+      <c r="I14" s="55"/>
     </row>
     <row r="15" spans="2:10">
-      <c r="C15" s="38" t="s">
+      <c r="C15" s="56" t="s">
         <v>64</v>
       </c>
-      <c r="D15" s="39"/>
-      <c r="E15" s="40"/>
-      <c r="G15" s="38" t="s">
+      <c r="D15" s="57"/>
+      <c r="E15" s="58"/>
+      <c r="G15" s="56" t="s">
         <v>65</v>
       </c>
-      <c r="H15" s="39"/>
-      <c r="I15" s="40"/>
+      <c r="H15" s="57"/>
+      <c r="I15" s="58"/>
     </row>
     <row r="16" spans="2:10">
-      <c r="C16" s="38" t="s">
+      <c r="C16" s="56" t="s">
         <v>66</v>
       </c>
-      <c r="D16" s="39"/>
-      <c r="E16" s="40"/>
-      <c r="G16" s="38" t="s">
+      <c r="D16" s="57"/>
+      <c r="E16" s="58"/>
+      <c r="G16" s="56" t="s">
         <v>67</v>
       </c>
-      <c r="H16" s="39"/>
-      <c r="I16" s="40"/>
+      <c r="H16" s="57"/>
+      <c r="I16" s="58"/>
     </row>
     <row r="17" spans="3:9">
-      <c r="C17" s="38"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="40"/>
-      <c r="G17" s="38" t="s">
+      <c r="C17" s="56"/>
+      <c r="D17" s="57"/>
+      <c r="E17" s="58"/>
+      <c r="G17" s="56" t="s">
         <v>68</v>
       </c>
-      <c r="H17" s="39"/>
-      <c r="I17" s="40"/>
+      <c r="H17" s="57"/>
+      <c r="I17" s="58"/>
     </row>
     <row r="18" spans="3:9">
-      <c r="C18" s="41"/>
-      <c r="D18" s="42"/>
-      <c r="E18" s="43"/>
-      <c r="G18" s="41"/>
-      <c r="H18" s="42"/>
-      <c r="I18" s="43"/>
+      <c r="C18" s="65"/>
+      <c r="D18" s="66"/>
+      <c r="E18" s="67"/>
+      <c r="G18" s="65"/>
+      <c r="H18" s="66"/>
+      <c r="I18" s="67"/>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="G16:I16"/>
     <mergeCell ref="B1:J3"/>
     <mergeCell ref="C13:E13"/>
     <mergeCell ref="G13:I13"/>
@@ -3432,16 +3393,6 @@
     <mergeCell ref="C10:E10"/>
     <mergeCell ref="G10:I11"/>
     <mergeCell ref="C11:E11"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="G17:I17"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="G16:I16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3472,47 +3423,47 @@
     </row>
     <row r="2" spans="1:10" ht="40.049999999999997" customHeight="1">
       <c r="A2" s="28"/>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="41" t="s">
         <v>149</v>
       </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
       <c r="H2" s="28"/>
       <c r="I2" s="28"/>
     </row>
     <row r="3" spans="1:10" ht="40.049999999999997" customHeight="1">
       <c r="A3" s="28"/>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
       <c r="H3" s="28"/>
       <c r="I3" s="28"/>
     </row>
     <row r="4" spans="1:10" ht="40.049999999999997" customHeight="1">
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
+      <c r="B4" s="41"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
     </row>
     <row r="5" spans="1:10" ht="36" customHeight="1"/>
     <row r="6" spans="1:10" ht="36" customHeight="1">
-      <c r="B6" s="57" t="s">
+      <c r="B6" s="69" t="s">
         <v>69</v>
       </c>
-      <c r="C6" s="58"/>
-      <c r="D6" s="58"/>
-      <c r="E6" s="58"/>
-      <c r="F6" s="59"/>
-    </row>
-    <row r="7" spans="1:10" ht="36" customHeight="1">
+      <c r="C6" s="70"/>
+      <c r="D6" s="70"/>
+      <c r="E6" s="70"/>
+      <c r="F6" s="71"/>
+    </row>
+    <row r="7" spans="1:10" ht="21.6" customHeight="1">
       <c r="B7" s="15" t="s">
         <v>70</v>
       </c>
@@ -3530,27 +3481,27 @@
       </c>
     </row>
     <row r="8" spans="1:10" s="29" customFormat="1" ht="21.6" customHeight="1">
-      <c r="B8" s="66" t="s">
+      <c r="B8" s="72" t="s">
         <v>129</v>
       </c>
-      <c r="C8" s="67"/>
-      <c r="D8" s="67"/>
-      <c r="E8" s="67"/>
-      <c r="F8" s="68"/>
-      <c r="H8" s="73"/>
-      <c r="I8" s="77" t="s">
+      <c r="C8" s="73"/>
+      <c r="D8" s="73"/>
+      <c r="E8" s="73"/>
+      <c r="F8" s="74"/>
+      <c r="H8" s="36"/>
+      <c r="I8" s="68" t="s">
         <v>229</v>
       </c>
-      <c r="J8" s="39"/>
+      <c r="J8" s="57"/>
     </row>
     <row r="9" spans="1:10" ht="36" customHeight="1">
-      <c r="B9" s="72">
+      <c r="B9" s="35">
         <v>2</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="D9" s="69" t="s">
+      <c r="D9" s="32" t="s">
         <v>221</v>
       </c>
       <c r="E9" s="15" t="s">
@@ -3559,20 +3510,20 @@
       <c r="F9" s="15">
         <v>3</v>
       </c>
-      <c r="H9" s="74"/>
-      <c r="I9" s="77" t="s">
+      <c r="H9" s="37"/>
+      <c r="I9" s="68" t="s">
         <v>230</v>
       </c>
-      <c r="J9" s="39"/>
+      <c r="J9" s="57"/>
     </row>
     <row r="10" spans="1:10" ht="36" customHeight="1">
-      <c r="B10" s="72">
+      <c r="B10" s="35">
         <v>3</v>
       </c>
-      <c r="C10" s="70" t="s">
+      <c r="C10" s="33" t="s">
         <v>112</v>
       </c>
-      <c r="D10" s="69" t="s">
+      <c r="D10" s="32" t="s">
         <v>222</v>
       </c>
       <c r="E10" s="15" t="s">
@@ -3581,54 +3532,54 @@
       <c r="F10" s="15">
         <v>2</v>
       </c>
-      <c r="H10" s="75"/>
-      <c r="I10" s="77" t="s">
+      <c r="H10" s="38"/>
+      <c r="I10" s="68" t="s">
         <v>231</v>
       </c>
-      <c r="J10" s="39"/>
+      <c r="J10" s="57"/>
     </row>
     <row r="11" spans="1:10" ht="36" customHeight="1">
-      <c r="B11" s="72">
+      <c r="B11" s="35">
         <v>2</v>
       </c>
-      <c r="C11" s="70" t="s">
+      <c r="C11" s="33" t="s">
         <v>115</v>
       </c>
-      <c r="D11" s="69" t="s">
+      <c r="D11" s="32" t="s">
         <v>223</v>
       </c>
-      <c r="E11" s="70" t="s">
+      <c r="E11" s="33" t="s">
         <v>78</v>
       </c>
       <c r="F11" s="15">
         <v>3</v>
       </c>
-      <c r="H11" s="76"/>
-      <c r="I11" s="77" t="s">
+      <c r="H11" s="39"/>
+      <c r="I11" s="68" t="s">
         <v>232</v>
       </c>
-      <c r="J11" s="39"/>
+      <c r="J11" s="57"/>
     </row>
     <row r="12" spans="1:10" s="29" customFormat="1" ht="21.6" customHeight="1">
-      <c r="B12" s="66" t="s">
+      <c r="B12" s="72" t="s">
         <v>133</v>
       </c>
-      <c r="C12" s="67"/>
-      <c r="D12" s="67"/>
-      <c r="E12" s="67"/>
-      <c r="F12" s="68"/>
+      <c r="C12" s="73"/>
+      <c r="D12" s="73"/>
+      <c r="E12" s="73"/>
+      <c r="F12" s="74"/>
     </row>
     <row r="13" spans="1:10" ht="36" customHeight="1">
-      <c r="B13" s="72">
+      <c r="B13" s="35">
         <v>2</v>
       </c>
-      <c r="C13" s="70" t="s">
+      <c r="C13" s="33" t="s">
         <v>76</v>
       </c>
-      <c r="D13" s="70" t="s">
+      <c r="D13" s="33" t="s">
         <v>224</v>
       </c>
-      <c r="E13" s="70" t="s">
+      <c r="E13" s="33" t="s">
         <v>78</v>
       </c>
       <c r="F13" s="15">
@@ -3636,16 +3587,16 @@
       </c>
     </row>
     <row r="14" spans="1:10" ht="36" customHeight="1">
-      <c r="B14" s="72">
+      <c r="B14" s="35">
         <v>1</v>
       </c>
-      <c r="C14" s="70" t="s">
+      <c r="C14" s="33" t="s">
         <v>77</v>
       </c>
-      <c r="D14" s="70" t="s">
+      <c r="D14" s="33" t="s">
         <v>225</v>
       </c>
-      <c r="E14" s="70" t="s">
+      <c r="E14" s="33" t="s">
         <v>78</v>
       </c>
       <c r="F14" s="15">
@@ -3653,25 +3604,25 @@
       </c>
     </row>
     <row r="15" spans="1:10" s="29" customFormat="1" ht="21.6" customHeight="1">
-      <c r="B15" s="66" t="s">
+      <c r="B15" s="72" t="s">
         <v>136</v>
       </c>
-      <c r="C15" s="67"/>
-      <c r="D15" s="67"/>
-      <c r="E15" s="67"/>
-      <c r="F15" s="68"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="73"/>
+      <c r="E15" s="73"/>
+      <c r="F15" s="74"/>
     </row>
     <row r="16" spans="1:10" ht="36" customHeight="1">
-      <c r="B16" s="72">
+      <c r="B16" s="35">
         <v>1</v>
       </c>
-      <c r="C16" s="70" t="s">
+      <c r="C16" s="33" t="s">
         <v>80</v>
       </c>
-      <c r="D16" s="70" t="s">
+      <c r="D16" s="33" t="s">
         <v>226</v>
       </c>
-      <c r="E16" s="70" t="s">
+      <c r="E16" s="33" t="s">
         <v>116</v>
       </c>
       <c r="F16" s="15">
@@ -3679,34 +3630,34 @@
       </c>
     </row>
     <row r="17" spans="2:8" ht="36" customHeight="1">
-      <c r="B17" s="72">
+      <c r="B17" s="35">
         <v>1</v>
       </c>
-      <c r="C17" s="70" t="s">
+      <c r="C17" s="33" t="s">
         <v>113</v>
       </c>
-      <c r="D17" s="70" t="s">
+      <c r="D17" s="33" t="s">
         <v>227</v>
       </c>
-      <c r="E17" s="70" t="s">
+      <c r="E17" s="33" t="s">
         <v>116</v>
       </c>
       <c r="F17" s="15">
         <v>3</v>
       </c>
-      <c r="H17" s="71"/>
+      <c r="H17" s="34"/>
     </row>
     <row r="18" spans="2:8" ht="36" customHeight="1">
-      <c r="B18" s="72">
+      <c r="B18" s="35">
         <v>1</v>
       </c>
-      <c r="C18" s="70" t="s">
+      <c r="C18" s="33" t="s">
         <v>114</v>
       </c>
-      <c r="D18" s="70" t="s">
+      <c r="D18" s="33" t="s">
         <v>228</v>
       </c>
-      <c r="E18" s="70" t="s">
+      <c r="E18" s="33" t="s">
         <v>116</v>
       </c>
       <c r="F18" s="15">
@@ -3723,28 +3674,28 @@
     <row r="20" spans="2:8" ht="19.95" customHeight="1"/>
   </sheetData>
   <mergeCells count="9">
+    <mergeCell ref="B2:G4"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B15:F15"/>
     <mergeCell ref="I8:J8"/>
     <mergeCell ref="I9:J9"/>
     <mergeCell ref="I10:J10"/>
     <mergeCell ref="I11:J11"/>
     <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B2:G4"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B15:F15"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <conditionalFormatting sqref="B9:B11 B13:B14 B16:B18">
-    <cfRule type="cellIs" dxfId="6" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="equal">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
       <formula>2</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3767,35 +3718,35 @@
   <sheetData>
     <row r="1" spans="1:9" s="21" customFormat="1" ht="40.049999999999997" customHeight="1">
       <c r="A1" s="28"/>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="41" t="s">
         <v>149</v>
       </c>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
       <c r="H1" s="28"/>
       <c r="I1" s="28"/>
     </row>
     <row r="2" spans="1:9" s="21" customFormat="1" ht="40.049999999999997" customHeight="1">
       <c r="A2" s="28"/>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
+      <c r="B2" s="41"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
       <c r="H2" s="28"/>
       <c r="I2" s="28"/>
     </row>
     <row r="3" spans="1:9" s="21" customFormat="1" ht="40.049999999999997" customHeight="1">
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
     </row>
     <row r="4" spans="1:9" ht="28.8">
       <c r="A4" s="22" t="s">
@@ -5104,18 +5055,18 @@
       </c>
     </row>
     <row r="4" spans="2:10">
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36" t="s">
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+      <c r="G4" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="H4" s="36"/>
-      <c r="I4" s="36"/>
-      <c r="J4" s="36"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="47"/>
+      <c r="J4" s="47"/>
     </row>
     <row r="5" spans="2:10" ht="28.8">
       <c r="B5" s="4" t="s">
@@ -5147,16 +5098,16 @@
       </c>
     </row>
     <row r="6" spans="2:10" ht="57.6">
-      <c r="B6" s="60" t="s">
+      <c r="B6" s="75" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="60" t="s">
+      <c r="C6" s="75" t="s">
         <v>38</v>
       </c>
-      <c r="D6" s="60" t="s">
+      <c r="D6" s="75" t="s">
         <v>39</v>
       </c>
-      <c r="E6" s="60" t="s">
+      <c r="E6" s="75" t="s">
         <v>40</v>
       </c>
       <c r="F6" s="5">
@@ -5176,10 +5127,10 @@
       </c>
     </row>
     <row r="7" spans="2:10" ht="72">
-      <c r="B7" s="61"/>
-      <c r="C7" s="61"/>
-      <c r="D7" s="61"/>
-      <c r="E7" s="61"/>
+      <c r="B7" s="76"/>
+      <c r="C7" s="76"/>
+      <c r="D7" s="76"/>
+      <c r="E7" s="76"/>
       <c r="F7" s="5">
         <v>2</v>
       </c>
@@ -5197,10 +5148,10 @@
       </c>
     </row>
     <row r="8" spans="2:10" ht="43.2">
-      <c r="B8" s="61"/>
-      <c r="C8" s="61"/>
-      <c r="D8" s="61"/>
-      <c r="E8" s="61"/>
+      <c r="B8" s="76"/>
+      <c r="C8" s="76"/>
+      <c r="D8" s="76"/>
+      <c r="E8" s="76"/>
       <c r="F8" s="5">
         <v>3</v>
       </c>
@@ -5218,10 +5169,10 @@
       </c>
     </row>
     <row r="9" spans="2:10">
-      <c r="B9" s="62"/>
-      <c r="C9" s="62"/>
-      <c r="D9" s="62"/>
-      <c r="E9" s="62"/>
+      <c r="B9" s="77"/>
+      <c r="C9" s="77"/>
+      <c r="D9" s="77"/>
+      <c r="E9" s="77"/>
       <c r="F9" s="5"/>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>

</xml_diff>